<commit_message>
data: pboat RSS universe 2026-07-27 [skip email]
</commit_message>
<xml_diff>
--- a/.github/scripts/output/universe-latest.xlsx
+++ b/.github/scripts/output/universe-latest.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Watchlist — by company" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI news — all'!$A$1:$K$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Watchlist — all'!$A$1:$M$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI news — all'!$A$1:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Watchlist — all'!$A$1:$M$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -532,10 +532,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>6.32</v>
+        <v>4.29</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -549,7 +549,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>Chinese CXMT DRAM doesn't look like the budget savior many were expecting — new modules enter the market, but prices still track the big three</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -559,15 +559,15 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>ai, nvidia, semiconductor, fab, ai infrastructure, ai partnership</t>
+          <t>semiconductor, fab, dram</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>10.1</v>
+        <v>10.5</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 13:55:35 +0000</t>
+          <t>Sun, 26 Jul 2026 13:25:30 +0000</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -577,16 +577,16 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.tomshardware.com/pc-components/dram/chinese-cxmt-dram-doesnt-look-like-the-budget-savior-many-were-expecting-new-modules-enter-the-market-but-prices-still-track-the-big-three</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>5.99</v>
+        <v>3.98</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -595,30 +595,30 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>OpenAI agent goes rogue and hacks popular AI community — left escape plans for future models inside the company's infrastructure</t>
+          <t>Hugging Face CEO calls for ‘radical transparency’ after ‘unprecedented’ OpenAI hack</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Tom's Hardware Premium equips you with world-class coverage and detailed insights into the evolving hardware landscape. Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive i</t>
+          <t>In Brief Posted: After OpenAI recently admitted that one of its models had breached the systems of AI platform Hugging Face , Hugging Face’s CEO Clem Delangue posted on X that he was flying to San Francisco to have “a little chat with that ‘rogue agent.’” Then, in a follow-up post on Saturday, Delangue outlined what he’d asked for from OpenAI. He said he called for “radical transparency,” asking O</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>openai, ai, semiconductor, fab</t>
+          <t>openai, autonomous</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 16:41:59 +0000</t>
+          <t>Sun, 26 Jul 2026 16:33:13 +0000</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -628,48 +628,48 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/openai-agent-goes-rogue-and-hacks-popular-ai-community-left-escape-plans-for-future-models-inside-the-companys-infrastructure</t>
+          <t>https://techcrunch.com/2026/07/26/hugging-face-ceo-calls-for-radical-transparency-after-unprecedented-openai-hack/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>5.72</v>
+        <v>3.8</v>
       </c>
       <c r="B4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>citation</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>channelnewsasia.com</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>AI cyberattacks mean we can't defend ourselves the same way as before: Singapore's founding cybersecurity chief</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Recent Searches Trending Topics CNA Explains China artificial intelligence Indonesia Malaysia podcasts Wellness Thailand Japan Get bite-sized news via a new cards interface. Give it a try. Click here to return to FAST Tap here to return to FAST FAST Singapore Recent Searches Trending Topics CNA Explains China artificial intelligence Indonesia Malaysia podcasts Wellness Thailand Japan Advertisement</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>tomshardware.com</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Tech Industry Artificial Intelligence Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories News By Anton Shilov Published 10 hours ago A lot of money, little to no details. (Image credit: Nvidia) Share this article 0 Join the conversation Follow us Add us as a preferred source on Google Newsletter Subscribe to o</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>ai, nvidia, ai infrastructure, ai partnership</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>10.1</v>
-      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 13:55:35 GMT</t>
+          <t>Mon, 27 Jul 2026 06:00:00 +0800</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -679,16 +679,16 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.channelnewsasia.com/singapore/cybersecurity-csa-founding-chief-david-koh-ai-cyberattack-defend-6275631</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4.79</v>
+        <v>3.68</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -697,30 +697,30 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>OpenAI agent goes rogue and hacks popular AI community — left escape plans for future models inside the company's infrastructure</t>
+          <t>Making sense of the panic over Chinese AI</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Tech Industry Artificial Intelligence OpenAI agent goes rogue and hacks popular AI community — left escape plans for future models inside the company's infrastructure News By Anton Shilov Published 7 hours ago What a covert AI agent! (Image credit: OpenAI) Share this article 1 Join the conversation Follow us Add us as a preferred source on Google Newsletter Subscribe to our newsletter The rogue Op</t>
+          <t>Making sense of the panic over Chinese AI Anthony Ha 12:40 PM PDT · July 26, 2026 The launch of the latest AI model from a Chinese company — Moonshot AI’s Kimi — reignited debates around American competitiveness and open versus proprietary AI. While there was plenty of conversation on social media , it seems the debate is also happening behind the scenes in Washington, D.C., where OpenAI and Anthr</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>openai, ai</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>7.3</v>
+        <v>4.3</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 16:41:59 GMT</t>
+          <t>Sun, 26 Jul 2026 19:40:57 +0000</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -730,13 +730,13 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/openai-agent-goes-rogue-and-hacks-popular-ai-community-left-escape-plans-for-future-models-inside-the-companys-infrastructure</t>
+          <t>https://techcrunch.com/2026/07/26/making-sense-of-the-panic-over-chinese-ai/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>4.1</v>
+        <v>3.67</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>1</v>
@@ -748,17 +748,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>thansettakij.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>คอมพิวเตอร์ควอนตัม: เทคโนโลยีที่จะเปลี่ยนโลก หลังยุค AI</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Play คอมพิวเตอร์ควอนตัม: เทคโนโลยีที่จะเปลี่ยนโลก หลังยุค AI By ดร.เมทังกร เสริมสุข 26 ก.ค. 69 | 06:15 น. คอมพิวเตอร์ควอนตัม เทคโนโลยีที่จะเปลี่ยนโลก หลังยุค AI ก้าวต่อไปของเศรษฐกิจดิจิทัลโลก โดย รองศาสตราจารย์ ดร.มนตรี วิบูลยรัตน์ รองคณบดี วิทยาลัยการจัดการนวัตกรรมและอุตสาหกรรม สถาบันเทคโนโลยีพระจอมเกล้าเจ้าคุณทหารลาดกระบัง (สจล.) ตลอดหลายปีที่ผ่านมา โลกให้ความสนใจกับปัญญาประดิษฐ์ (Artificial Int</t>
+          <t>The homepage The Verge The Verge logo. Notifications Notifications Hamburger Navigation Button Navigation Drawer The Verge The Verge logo. Login / Sign Up close Close Light System Dark Subscribe Facebook Threads Instagram Youtube RSS Comments Drawer Notifications Comments Loading comments Getting the conversation ready... Tech Gadgets News Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -767,11 +767,11 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.7</v>
+        <v>4.4</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 23:15:00 GMT</t>
+          <t>2026-07-26T15:36:38-04:00</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -781,13 +781,13 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>https://www.thansettakij.com/blogs/columnist/neotech-forums/664938</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>3.86</v>
+        <v>3.35</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>1</v>
@@ -804,25 +804,25 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Grab an Nvidia RTX 5060 Ti gaming PC with Core Ultra 7 CPU and 32GB RAM for under $1,200 — Thermaltake's View u2660T-170 slashed by 33%</t>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive into our proprietary testing data and compare hardware with detailed benchmarks. Go beyond the headlines with expert repo</t>
+          <t>Tom's Hardware Premium equips you with world-class coverage and detailed insights into the evolving hardware landscape. Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive i</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>nvidia, amd</t>
+          <t>ai, nvidia</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>8.699999999999999</v>
+        <v>14</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 15:18:22 +0000</t>
+          <t>Sun, 26 Jul 2026 10:00:00 +0000</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -832,13 +832,13 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/pc-components/grab-an-nvidia-rtx-5060-ti-gaming-pc-with-core-ultra-7-cpu-and-32gb-ram-for-under-usd1-200-thermaltakes-view-u2660t-170-slashed-by-33-percent</t>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>3.77</v>
+        <v>3.33</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1</v>
@@ -850,46 +850,46 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>reuters.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Samsung Elec wins $200 billion Broadcom AI chip partnership, boosting foundry push</t>
+          <t>TechCrunch Mobility: Uber bets on its former CEO</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Samsung Elec wins $200 billion Broadcom AI chip partnership, boosting foundry push    Reuters</t>
+          <t>TechCrunch Mobility: Uber bets on its former CEO Kirsten Korosec 9:03 AM PDT · July 26, 2026 Welcome back to TechCrunch Mobility , your hub for the future of transportation and now, more than ever, the role AI is playing in it. To get this in your inbox, sign up here for free — just click TechCrunch Mobility ! Tesla kicked off earnings season — at least for this sector — and the shareholder letter</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>ai, chip</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>9.6</v>
+        <v>7.9</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 14:25:36 GMT</t>
+          <t>Sun, 26 Jul 2026 16:03:00 +0000</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>https://www.reuters.com/business/autos-transportation/samsung-elec-wins-200-billion-broadcom-ai-chip-partnership-boosting-foundry-push-2026-07-25/</t>
+          <t>https://techcrunch.com/2026/07/26/techcrunch-mobility-uber-bets-on-its-former-ceo/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>3.71</v>
+        <v>3.14</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>1</v>
@@ -901,30 +901,30 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>blognone.com</t>
+          <t>cnbc.com</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Anthropic ออก Claude Opus 5 บอกเก่งเทียบเท่า Fable 5 แต่ถูกกว่าครึ่งหนึ่ง</t>
+          <t>How AI wealth could be distributed to all Americans</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Anthropic อัปเดตโมเดลปัญญาประดิษฐ์รุ่น(เคย)บน Claude Opus 5 โดยคราวนี้เทียบกับ Fable 5 ที่เป็นโมเดลรุ่นบนสุดปัจจุบัน บอกว่ามีความฉลาดในการทำงานซับซ้อนใกล้เคียงกัน แต่ราคาใช้งานถูกกว่าครึ่งหนึ่ง Opus 5 มีความเก่งกว่าทุกหัวข้อเมื่อเทียบกับ Opus 4.8 ทั้งงานความรู้รอบตัว งานเขียนโค้ด ส่วนหัวข้อที่มักเจอการจำกัดใน Fable 5 อย่างเคมี-ชีววิทยา ก็ไม่มีปัญหาเรื่องนี้ เพราะโมเดลถูกควบคุมไว้แล้วในตอนฝึกฝนข้อม</t>
+          <t xml:space="preserve">WATCH LIVE THE BOTTOM LINE How AI wealth could be distributed to all Americans PUBLISHED SUN, JUL 26 2026 10:06 AM EDT Trevor Laurence Jockims WATCH LIVE KEY POINTS Bernie Sanders' recent proposal that the public should own half of artificial intelligence is unlikely to become policy anytime soon, but new models are being proposed to both regulate AI and create mechanisms for sharing trillions of </t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>anthropic, claude, ปัญญาประดิษฐ์, โมเดล</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>22.8</v>
+        <v>9.9</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 01:07:52 +0000</t>
+          <t>Sun, 26 Jul 2026 14:06:53 GMT</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -934,13 +934,13 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>https://www.blognone.com/node/151227</t>
+          <t>https://www.cnbc.com/amp/2026/07/26/how-can-ai-wealth-be-shared-with-all-americans.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>3.65</v>
+        <v>3.08</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1</v>
@@ -952,30 +952,30 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>One fallen power line exposed a growing AI data center problem. Here’s how to fix it.</t>
+          <t>Meta AI อัปเดตความสามารถ ช่วยวางแผน สรุปเนื้อหา ด้วยโมเดล Muse Spark 1.1</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>One fallen power line exposed a growing AI data center problem. Here’s how to fix it. Tim De Chant 6:05 AM PDT · July 25, 2026 A power line went down outside of Washington, DC, this week. Normally, the grid would only need a few seconds to recover from such an event. But this one took more than 10 minutes because more than 3 gigawatts of data centers stopped drawing power nearly simultaneously. Th</t>
+          <t>Meta AI แอปผู้ช่วย AI ของ Meta อัปเดตความสามารถใหม่หลังจากโมเดล [Muse Spark 1.1](Muse Spark 1.1) ออกมาเมื่อต้นเดือน โดยขยายความสามารถจากการเป็นแชทบอตถามตอบ ไปสู่ผู้ช่วยที่สามารถวางแผน คิด และให้ข้อมูลล่วงหน้าได้ ในอัปเดตนี้ผู้ใช้งานสามารถเปิดการเชื่อมต่อ Meta AI กับอีเมลและปฏิทิน เพื่อนำข้อมูลมาช่วยวางแผนหรือสรุปประเด็นต่าง ๆ เช่น สรุปเนื้อหาประจำวัน, วางแผนระยะยาวเช่นปรับปรุงบ้าน โดยสามารถค้นข้อม</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>ai, data center</t>
+          <t>ai, โมเดล</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>10.9</v>
+        <v>16.9</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 13:05:00 +0000</t>
+          <t>Sun, 26 Jul 2026 07:04:09 +0000</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -985,13 +985,13 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/one-fallen-power-line-exposed-a-growing-ai-data-center-problem-heres-how-to-fix-it/</t>
+          <t>https://www.blognone.com/node/151235</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>3.53</v>
+        <v>3.01</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1</v>
@@ -1003,17 +1003,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>theverge.com</t>
+          <t>aljazeera.com</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>What is the AI Kill Switch Act proposed in the US and how will it work?</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>The homepage The Verge The Verge logo. Notifications Notifications Hamburger Navigation Button Navigation Drawer The Verge The Verge logo. Login / Sign Up close Close Light System Dark Subscribe Facebook Threads Instagram Youtube RSS Comments Drawer Notifications Comments Loading comments Getting the conversation ready... Tech Business News Google basically confirms the Pixel 11 is getting a price</t>
+          <t>EXPLAINER News | Internet What is the AI Kill Switch Act proposed in the US and how will it work? US lawmakers introduce a bill aimed at giving the government power to order companies to shut down AI systems if they escape human control. Listen (5 mins) Save Click here to share on social media Share Add Al Jazeera on Google OpenAI CEO Sam Altman speaks during a panel discussion at the Technical Un</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1022,11 +1022,11 @@
         </is>
       </c>
       <c r="H11" s="2" t="n">
-        <v>5.8</v>
+        <v>11.3</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T14:13:36-04:00</t>
+          <t>Sun, 26 Jul 2026 12:40:54 GMT</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1036,13 +1036,13 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+          <t>https://www.aljazeera.com/news/2026/7/26/what-is-the-ai-kill-switch-act-proposed-in-the-us-and-how-will-it-work</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>1</v>
@@ -1054,46 +1054,46 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>www3.nhk.or.jp</t>
+          <t>tomshardware.com</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>การใช้งาน generative AI ในญี่ปุ่นเกินร้อยละ 50 เป็นครั้งแรก</t>
+          <t>XFX Radeon RX 9070 XT drops to its lowest price of the summer — save $90 on AMD's flagship RDNA 4 graphics card</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>การใช้งาน generative AI ในญี่ปุ่นเกินร้อยละ 50 เป็นครั้งแรก    nhk.or.jp</t>
+          <t>Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive into our proprietary testing data and compare hardware with detailed benchmarks. Go beyond the headlines with expert repo</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>ai, generative ai</t>
+          <t>amd</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>13.5</v>
+        <v>11.4</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 10:28:09 GMT</t>
+          <t>Sun, 26 Jul 2026 12:31:14 +0000</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE9hMm81TGx6eXVvdlZyd3F2NXNSbFF6UDJIVTZpNjFZWmlOSktBXzE0WlZhTFJIbTlDNnJ6aFB5N1FyX0dYUklJQW5IaTd5V19FZmVfVU56LWR2enJVcUlMRDlR?oc=5</t>
+          <t>https://www.tomshardware.com/pc-components/xfx-radeon-rx-9070-xt-drops-to-its-lowest-price-of-the-summer-save-usd90-on-amds-flagship-rdna-4-graphics-card</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>3.32</v>
+        <v>2.95</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1</v>
@@ -1105,30 +1105,30 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>tomshardware.com</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Librarians are hosting viral ‘Avoiding AI’ workshops for people who are fed up with Big Tech</t>
+          <t>3D-printed F-14 Tomcat uses an FPGA recreation of the ‘world’s first microprocessor' — CADC’s MP944 chip controls the fighter’s swing-wing system, among other things</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Librarians are hosting viral ‘Avoiding AI’ workshops for people who are fed up with Big Tech Amanda Silberling 9:00 AM PDT · July 25, 2026 “Everybody’s on their phone at my program!” jokes Charlie Bailey, a librarian in South Philadelphia. He’s just asked his audience to pull out their phones so that he can walk them through the steps of disabling Apple Intelligence and Gemini. Bailey stands at th</t>
+          <t>Tom's Hardware Premium equips you with world-class coverage and detailed insights into the evolving hardware landscape. Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive i</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>chip</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>8</v>
+        <v>11.9</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 16:00:00 +0000</t>
+          <t>Sun, 26 Jul 2026 12:05:00 +0000</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1138,13 +1138,13 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/librarians-are-hosting-viral-avoiding-ai-workshops-for-people-who-are-fed-up-with-big-tech/</t>
+          <t>https://www.tomshardware.com/pc-components/cpus/3d-printed-f-14-tomcat-uses-an-fpga-recreation-of-the-worlds-first-microprocessor-cadcs-mp944-chip-controls-the-fighters-swing-wing-system-among-other-things</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>3.29</v>
+        <v>2.72</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>1</v>
@@ -1156,30 +1156,30 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>www3.nhk.or.jp</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>'RAM Machine' case probably costs more than the entire build — Nvidia RTX 5060, Core Ultra 5 CPU, and 32GB DDR5-8200 RAM are hiding inside</t>
+          <t>บริษัทจากสหรัฐและเกาหลีใต้ลงนามข้อตกลงด้านปัญญาประดิษฐ์มูลค่า 950,000 ล้านดอลลาร์</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Jowi Morales is a writer and journalist covering the tech beat since 2021. However, he’s been interested in technology far earlier than that. He started discovering desktop computers when his father brought home a Windows 95 PC, but his first real experience working under the hood of the PC was when</t>
+          <t>บริษัทจากสหรัฐและเกาหลีใต้ลงนามข้อตกลงด้านปัญญาประดิษฐ์มูลค่า 950,000 ล้านดอลลาร์    nhk.or.jp</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>ปัญญาประดิษฐ์</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>8.4</v>
+        <v>14.3</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 15:34:57 +0000</t>
+          <t>Sun, 26 Jul 2026 09:42:56 GMT</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1189,13 +1189,13 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/desktops/gaming-pcs/ram-machine-case-probably-costs-more-than-the-entire-build-nvidia-rtx-5060-core-ultra-5-cpu-and-32gb-ddr5-8200-ram-are-hiding-inside</t>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE41RktZcHhGY2tiMHNsRzJDbERZcmpMTzZONHdvSjRiMldCaFlzbFlQSDMyckt6dTN4R3I0cWU2NEF4MUVQYjRmcFc0MzJFTHlEZjlXckc0T3N5M1VwNjRNZFF3?oc=5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>3.05</v>
+        <v>2.7</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>1</v>
@@ -1207,17 +1207,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>theregister.com</t>
+          <t>techsauce.co</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>How AI drove Shopify back to clean code</t>
+          <t>3 มุมจากผู้ลงมือทำ AI Transformation เมื่อ AI ไม่ใช่ซอฟต์แวร์สำเร็จรูป ที่ซื้อมาแล้วองค์กรจะเปลี่ยนได้เอง</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">E-commerce platform Shopify wants to make reading source code a thing again. And it has an unlikely ally for its back-to-the-roots approach: AI agents. The company is launching a new storefront theme for its customers, aka “merchants,” that it claims is completely understandable by anyone with even </t>
+          <t>ใน Session ที่ 3 ของงาน HOW Quarterly Public Session: Burning Platform Corporate Survival Guide in the Age of AI ในช่วง Panel Discussion ที่นำเอาผู้ลงมือจริงในอุตสาหกรรม IT Consultanting และ Solution มาร่วมแลกเปลี่ยนมุมมอง เสวนาโดย 3 ผู้บริหารชั้นนำ ได้แก่    คุณเล้ง ศิริวัฒน์ วงศ์จารุกร จาก MFEC  ค</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1226,11 +1226,11 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>10.9</v>
+        <v>14.5</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 15:06:00 +0200</t>
+          <t>Sun, 26 Jul 2026 16:29:21 +0700</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1240,13 +1240,13 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>https://www.theregister.com/devops/2026/07/25/how-ai-drove-shopify-back-to-clean-code/5277901</t>
+          <t>https://techsauce.co/ai/3-ai-corporate-survival-guide-how-quarterly</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>3.04</v>
+        <v>2.69</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>1</v>
@@ -1258,30 +1258,33 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>theguardian.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>The AI jobs apocalypse probably isn’t coming anytime soon</t>
+          <t>เว็บรับโฮสต์ซอฟต์แวร์ Codeberg แบนไม่รับโค้ดที่เขียนด้วย LLM บอกสิ้นเปลืองทรัพยากร</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>The AI jobs apocalypse probably isn’t coming anytime soon    The Guardian</t>
+          <t>เว็บรับโฮสต์ซอฟต์แวร์ Codeberg แบนไม่รับโค้ดที่เขียนด้วย LLM บอกสิ้นเปลืองทรัพยากร 
+     Body 
+                Codeberg บริการโฮสต์ซอร์สโค้ดสายโอเพนซอร์ส ( ข่าวเก่า ) ประกาศปิดรับโค้ดที่เขียนด้วย AI และ LLM ไม่ให้เข้ามาฝากในระบบ 
+ ปัญหาเรื่องโค้ดที่สร้างด้วย AI/LLM มีปริมาณมากจนรับไม่ไหว  ส่งผล</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>ai, llm</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 13:01:00 GMT</t>
+          <t>Sun, 26 Jul 2026 02:58:45 +0000</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1291,13 +1294,13 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxOTlRPeHY4ZnZBa010WDFSS1p4YUxWNzdVRWo3X0g0Vk5LUEdFcjBsbnBMWTAzdG9jS0FUMTFKNkNsSnJnMTlNR1BoVkhYQy1EZmN2ZV8yWVJKbTFVTWJwZ2F2TjFLcU1OSlc4WEt6dW14QU1LUkFZVnlVUEpmVE93bGlkNEhqajRR?oc=5</t>
+          <t>https://www.blognone.com/node/151234</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>2.94</v>
+        <v>2.51</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>1</v>
@@ -1309,30 +1312,30 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>cnbc.com</t>
+          <t>mgronline.com</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Analysis: A powerful new coalition of AI skeptics is coalescing right in Trump's blind spot</t>
+          <t>OpenAI ยอมรับ AI หลุดจากห้องทดสอบ แฮ็กระบบ Hugging Face ได้เอง</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Analysis: A powerful new coalition of AI skeptics is coalescing right in Trump's blind spot    CNBC</t>
+          <t>OpenAI ยอมรับ AI หลุดจากห้องทดสอบ แฮ็กระบบ Hugging Face ได้เอง    ผู้จัดการออนไลน์</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>openai, ai</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>12</v>
+        <v>22.8</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 12:00:02 GMT</t>
+          <t>Sun, 26 Jul 2026 01:09:00 GMT</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1342,13 +1345,13 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE13ZHNTM1NUV0Jyd1ZlTmJpYWNFQmZ6dUd6N3JlVC1scVpSNUN2N0xRWUd0ZmVWSlFCZGd1MHZIYzBzeXQ2MjVGNzhtZ2RVVEVsUDBSV0Jwa0JieUY3SjJXcmp6S0R1WnZNLWNoZVRHYk5zdWZF0gF6QVVfeXFMUFY0a1BQZVRCWTMxWl9sNVg2U0JHaUlNTGNVb3g4VnJueXFMV195VWo0bWkxOFF6Z19ZanBFS3haTTM0ajJEYTZSMDN1Qno5ZUVXU2NyaVQ4Tm9pV1BIcDh6RHE0b3NQYUdHT2lmVldPRnlaU2IyelNNX0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9lekV0bjdZNlNXZzdFQ183Z3Z0UVd5U3pCbUhFY3BHdThpSW1lRm4ta1VzTFI1WS1PVTFfTGNyUWRCVGhlVFBpa3JvTlQ2Znp4NUE0YkdaV0xsY1dVX2NMYg?oc=5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>2.9</v>
+        <v>2.38</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>1</v>
@@ -1360,30 +1363,30 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>bangkokbiznews.com</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Microsoft shipped a native Xbox 360 emulator with its new backwards-compatible releases on PC — modders quickly got 360 games running with minor tweaks</t>
+          <t>กูรูชี้หุ้นโลกครึ่งปีหลังยังไปต่อ แต่กำไรเริ่มจำกัด ชูสหรัฐฯ-เกาหลีใต้เด่น รับเมกะเทรนด์ AI</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Hassam is a lifelong PC gamer and tech enthusiast with over five years of experience in PC hardware journalism. His passion began in childhood when he rescued a discarded Pentium 4 processor, straightening its pins with a kitchen knife to revive a Dell Dimension 2400 at the age of seven. Since then,</t>
+          <t>กูรูชี้หุ้นโลกครึ่งปีหลังยังไปต่อ แต่กำไรเริ่มจำกัด ชูสหรัฐฯ-เกาหลีใต้เด่น รับเมกะเทรนด์ AI    bangkokbiznews</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>amd</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>12.5</v>
+        <v>17.9</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 11:30:00 +0000</t>
+          <t>Sun, 26 Jul 2026 06:04:41 GMT</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1393,48 +1396,48 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/video-games/xbox/microsoft-shipped-a-native-xbox-360-emulator-with-its-new-backwards-compatible-releases-on-pc-modders-quickly-got-360-games-running-with-minor-tweaks</t>
+          <t>https://news.google.com/rss/articles/CBMiYkFVX3lxTE1BT2NZbXd6OXZLU0dXaXlqZ0hJVjVqUDMyR3NTUWhmNDJiVlZsNFVaQXpoRE1ER2JMdFRoZTd1Tk13WGptOEZlMnZScm5GNmVQMF9DeVByVzFSZjRheHpTaGhB?oc=5</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>2.88</v>
+        <v>2.34</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>citation</t>
+          <t>screening</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>engadget.com</t>
+          <t>bloomberg.com</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>OpenAI's rogue agent went on a hacking spree that lasted days, Reuters says</t>
+          <t>Big Tech Earnings Slam Into a Market in Revolt Over AI Spending</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Reuters reports that the OpenAI agent that hacked Hugging Face had been free for a week before the company noticed.</t>
+          <t>Big Tech Earnings Slam Into a Market in Revolt Over AI Spending    Bloomberg.com</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>12.7</v>
+        <v>11</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 11:15:05 +0000</t>
+          <t>Sun, 26 Jul 2026 13:00:00 GMT</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1444,13 +1447,13 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>https://www.engadget.com/2223141/openai-rogue-agent-days-hacking-spree-reuters/</t>
+          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOLTlyY0loRTZCSWVPcmtFSW0zWUF3Tmc3ekN1ajNfMkZYZThOTFJLaDNxdUNCaVNyb0ZHQTB4b01QREFXVXcwZkdRYUExUkdoOFRPMHdXelRNRTZ5ZV9XM0twdi1neDZvWmdEZjFHdmxiZXJHSWpiWDN5WWFmVFRWY0xDdmtLN25HSEloYXpjeUFqRjlZMmhQbWtzSnZ3amRjeEEtODlfa1BSS3Z6bnFUVE43TkE?oc=5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>2.79</v>
+        <v>2.2</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>1</v>
@@ -1462,30 +1465,30 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>bangkokbiznews.com</t>
+          <t>thairath.co.th</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>'ชนาพัฒน์' ดึง AI ขับเคลื่อนดีไซน์ เปิด Open House สิงหาคม นี้</t>
+          <t>รู้จัก “เช แท-วอน” ผู้สืบทอดแชโบล พลิกชะตา SK Hynix จากเกือบเจ๊งสู่ราชา HBM มูลค่าเฉียดล้านล้าน</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>'ชนาพัฒน์' ดึง AI ขับเคลื่อนดีไซน์ เปิด Open House สิงหาคม นี้    bangkokbiznews</t>
+          <t>รู้จัก “เช แท-วอน” ผู้สืบทอดแชโบล พลิกชะตา SK Hynix จากเกือบเจ๊งสู่ราชา HBM มูลค่าเฉียดล้านล้าน    Thairath.co.th</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>hbm</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>13.6</v>
+        <v>19.8</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 10:20:00 GMT</t>
+          <t>Sun, 26 Jul 2026 04:11:56 GMT</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1495,13 +1498,13 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1aNnVxZHhOdGZFeFJyLTJPZXNpb3JydnktNnRIbHhtWU45WGwtRFlMc3V2ZmJjVG9CLVVFNmZ5em93VFV5Rm41akVxWEVURXhKV21MY1NLcVJjdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPeFhLa1pobWE2NGoyU0lJNmV6YXJxMFVPQ08zd1MwbkJHWWpZcXVJSDdfRHNzaDdEakJKNlhyYVYtRW1IRG90SFBpXzktRVFEZklQYTBrYTlvYTZpNkJHenRDLS1wZkJWdEJtNmgwVC1VRXhSMTFPelpjRENFdWJSVzM1dw?oc=5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>2.78</v>
+        <v>2.03</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>1</v>
@@ -1513,17 +1516,19 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>theregister.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Anti-AI open source has an enemy in common, but almost nothing else</t>
+          <t>ลีกเบสบอลสหรัฐ สั่งห้ามใช้ AI ช่วยวางแผนในระหว่างแข่งขัน หลังพบแนวโน้มมีมากขึ้น</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>OPINION Linux now being officially not anti-AI might be good news for projects that are explicitly anti-AI, but we foresee problems with conflict over where the money and development effort come from. A couple of weeks ago, reluctant geek superstar Linus Torvalds declared that Linux is not an anti-A</t>
+          <t>ลีกเบสบอลสหรัฐ สั่งห้ามใช้ AI ช่วยวางแผนในระหว่างแข่งขัน หลังพบแนวโน้มมีมากขึ้น 
+     Body 
+                มีประเด็นน่าสนใจเกี่ยวกับ AI และแวดวงกีฬาเมื่อ MLB ผู้จัดการแข่งขันลีกเบสบอลในสหรัฐ ออกกฎห้ามแต่ละทีมใช้ AI ผ่านแท็บเล็ตขณะนั่งอยู่ในสนาม เพื่อช่วยการตัดสินใจและปรับกลยุทธ์ ในระหว่างการแข</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1532,11 +1537,11 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>13.7</v>
+        <v>21.6</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 12:17:00 +0200</t>
+          <t>Sun, 26 Jul 2026 02:20:47 +0000</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1546,13 +1551,13 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>https://www.theregister.com/ai-and-ml/2026/07/25/anti-ai-open-source-has-an-enemy-in-common-but-almost-nothing-else/5278275</t>
+          <t>https://www.blognone.com/node/151233</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>2.78</v>
+        <v>1.94</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>1</v>
@@ -1564,17 +1569,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>bangkokbiznews.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>‘ดีอี’ วางหมาก AI ดันไทยสู่ศูนย์กลางภูมิภาค ชู ‘ธรรมาภิบาล-โครงสร้างพื้นฐาน-คน’</t>
+          <t>Monday.com is the latest tech company to blame AI for layoffs — here are 20 others</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>‘ดีอี’ วางหมาก AI ดันไทยสู่ศูนย์กลางภูมิภาค ชู ‘ธรรมาภิบาล-โครงสร้างพื้นฐาน-คน’    bangkokbiznews</t>
+          <t>A running look — in reverse chronological order — at the bigger tech companies that have announced significant layoffs this year with AI as a stated factor.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1583,11 +1588,11 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>13.7</v>
+        <v>22.5</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 10:17:00 GMT</t>
+          <t>Sun, 26 Jul 2026 01:30:00 +0000</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1597,13 +1602,13 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1heWpqY09tLWtvTjBqSldHdS1UdzRDUEplQW1qU01tWTJPZVZEQzZyUzl3eW5maW1iVlc2bXNXcUp4UzFaWUg5aWRQRmNCd0ZQMDhqeWtyM2pKQQ?oc=5</t>
+          <t>https://techcrunch.com/2026/07/25/the-running-list-major-tech-layoffs-in-2026-where-employers-cited-ai/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>2.77</v>
+        <v>1.94</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>1</v>
@@ -1615,30 +1620,33 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>techsauce.co</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>ทำความรู้จัก Yang Zhilin ผู้ก่อตั้ง Moonshot AI จากนักวิจัยที่ฝันอยากเป็นร็อกสตาร์ สู่เจ้าของ Kimi K3</t>
+          <t>Meta ออกแอพแยก Seller สำหรับผู้ขายสินค้าบน Facebook Marketpace</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>ที่สำนักงานของ Moonshot AI ในย่านจงกวนชุน กรุงปักกิ่ง ห้องประชุมถูกตั้งชื่อตามวงร็อกในตำนานอย่าง Rolling Stones และ Led Zeppelin ขณะที่ชื่อบริษัทในภาษาจีน 月之暗面 แปลตรงตัวว่า 'ด้านมืดของดวงจันทร์' ซึ่งหยิบมาจากอัลบั้ม The Dark Side of the Moon ของวง Pink Floyd โดยตรง เบื้องหลังรายละเอียดเหล่านี้คือชาย</t>
+          <t>Meta ออกแอพแยก Seller สำหรับผู้ขายสินค้าบน Facebook Marketpace 
+     Body 
+                Meta ออกแอพมือถือใหม่ชื่อ  Seller  เป็นแอพแยกสำหรับผู้ขายใน Facebook Marketplace 
+ Meta ให้เหตผลของการแยกแอพว่า ต้องการให้พื้นที่เฉพาะแก่ผู้ขาย มีเครื่องมืออำนวยความสะดวก เช่น สร้างรายละเอียดสินค้าด้วย AI</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>ai, ปัญญาประดิษฐ์</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>20.1</v>
+        <v>22.5</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 10:49:53 +0700</t>
+          <t>Sun, 26 Jul 2026 01:30:36 +0000</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1648,13 +1656,13 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>https://techsauce.co/basedon/yang-zhilin-moonshot-ai-kimi-k3</t>
+          <t>https://www.blognone.com/node/151231</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>2.75</v>
+        <v>1.85</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>1</v>
@@ -1666,17 +1674,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>cbc.ca</t>
+          <t>bangkokbiznews.com</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>What’s it like having an AI boyfriend? 2 Waterloo researchers decided to find out</t>
+          <t>สหรัฐฯ เดินหมากตัวที่ 4 ใช้ AI ทำ Dollarization</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>What’s it like having an AI boyfriend? 2 Waterloo researchers decided to find out    CBC</t>
+          <t>สหรัฐฯ เดินหมากตัวที่ 4 ใช้ AI ทำ Dollarization    bangkokbiznews</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1685,11 +1693,11 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>14</v>
+        <v>23.5</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 10:00:00 GMT</t>
+          <t>Sun, 26 Jul 2026 00:30:00 GMT</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1699,267 +1707,12 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1gFBVV95cUxNalJDcHlhNHhfZFFUVXNJZTBDeVcxSnAwSlU3aHpKN3hUWmFaQ2I4VVdsUUhnTm5JYS1ielp5SUFlcUd1Y0kwRVZIM3B3TE9DamJMRUpvb1hRbFBLeG9BVnBvSU9NeFZ2MEJ0WEJhQ0J0U1o4blRKdERwNHRydEZpLW02M002N2hGd3VfX0RZbGF4V3RTT3I2ZFFaUkJzQUh4TjJJMGhWSVB1Uk03ZTdvTEJQRjVLamdJRWlETEkwdG1IYldDWFNRRGZBMUJKTjNwMU4tTUdR?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>2.69</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>bangkokbiznews.com</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>‘Nvidia’ ทุ่มพันล้าน ผนึก ‘Naver-SK’ สร้างฮับ ‘ดาต้าเซ็นเตอร์’ ชี้เป็นยุคทองเกาหลีใต้</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>‘Nvidia’ ทุ่มพันล้าน ผนึก ‘Naver-SK’ สร้างฮับ ‘ดาต้าเซ็นเตอร์’ ชี้เป็นยุคทองเกาหลีใต้    bangkokbiznews</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>nvidia, ดาต้าเซ็นเตอร์</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 03:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE5XVEprNmRkRlIzem5TdXV3WVBTSGhhdmhlaUM4b2RoWU1CanpPRzBKci1oMG5BQXB2dkJTSjhkZUl2a1VVWjdGZUhyVnNwU1pxMFJVOFNvYXpiYTRRZXVCVDBkUnI?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>techcrunch.com</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>I tried out OpenAI’s new AI keypad — which will be fun for some coders and slightly mystifying to everyone else</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>OpenAI's fancy new AI keypad will be a lot of fun for some, while many others are probably not going to touch it.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>openai, ai</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 00:23:11 +0000</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>https://techcrunch.com/2026/07/24/i-tried-out-openais-new-ai-keypad-which-will-be-fun-for-coders-and-slightly-mystifying-to-everyone-else/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>koreaherald.com</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Korea, US tech giants set sights on $950 billion in chip partnerships: Seoul</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Korea, US tech giants set sights on $950 billion in chip partnerships: Seoul    The Korea Herald</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>chip</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 05:12:38 GMT</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE8xWDZKSkU1TXRqU28zS3k3OVRaQkh2T3ZNa1ZQZHRfUjRSX1RDSDRWVnZWeEtvODNhdE1fenBlNGlNMi01SUhtRTlCTlNtU3MwaEp3ZHVBbw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>matichon.co.th</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>SSVIT จัดโครงการ ครูพันธุ์ใหม่ หัวใจนวัตกรรม ครั้งที่ 1 : AI for Education เพื่อผู้เรียนแห่งอนาคต</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>SSVIT จัดโครงการ ครูพันธุ์ใหม่ หัวใจนวัตกรรม ครั้งที่ 1 : AI for Education เพื่อผู้เรียนแห่งอนาคต    มติชนออนไลน์</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>ai</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 04:59:38 GMT</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE9fMFNLbmlsdUFRY010VW5iVW1SQVlmM2s3eFZkREQ4S2dwS1hiMEs1dGlXMWphbHh6dEswdkFpVUdWQ3pwZzV5c2I4cEFJZTVEQlp3UU5WSjRVU242Um1qYnZLSXZRZw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>thansettakij.com</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>‘ดาวโจนส์’ ปิดตลาดบวก 235 จุด-Nasdaq ร่วง จับตาหุ้น AI สัปดาห์หน้า</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>‘ดาวโจนส์’ ปิดตลาดบวก 235 จุด-Nasdaq ร่วง จับตาหุ้น AI สัปดาห์หน้า    thansettakij</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>ai</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 01:18:00 GMT</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE9kdFVBSGM3Wnk0c04tTnFIUFZwM1BBU21nTlFlYWpvTWlwekF2QmZYckxlZlV0M3pMRlotT2lSZk9sd21XUWVocnFScVotYTBTS0VDVDln?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE43dUhRd2xleDVzWFB1YUhhU0lMS21NbTc0ekJoWVFCZGprcXA4SEFGTEY0NUZRTEpBX2hrRHVLbUpkZWFONFdNWHY3Yy1qUmJlaG5TRlBmSmg4cklnYXdoWGVpTEk5VXU3VW5oZ3J5WQ?oc=5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K29"/>
+  <autoFilter ref="A1:K24"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
@@ -1984,11 +1737,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2060,25 +1808,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>6.32</v>
+        <v>4.29</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>rec1.32+sig3.0+src1.2+corr0.8</t>
+          <t>rec1.29+sig1.8+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>Chinese CXMT DRAM doesn't look like the budget savior many were expecting — new modules enter the market, but prices still track the big three</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ai, nvidia, semiconductor, fab, ai infrastructure, ai partnership</t>
+          <t>semiconductor, fab, dram</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -2087,7 +1835,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.tomshardware.com/pc-components/dram/chinese-cxmt-dram-doesnt-look-like-the-budget-savior-many-were-expecting-new-modules-enter-the-market-but-prices-still-track-the-big-three</t>
         </is>
       </c>
     </row>
@@ -2096,34 +1844,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>5.99</v>
+        <v>3.98</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>rec1.59+sig2.4+src1.2+corr0.8</t>
+          <t>rec1.58+sig1.2+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>OpenAI agent goes rogue and hacks popular AI community — left escape plans for future models inside the company's infrastructure</t>
+          <t>Hugging Face CEO calls for ‘radical transparency’ after ‘unprecedented’ OpenAI hack</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>openai, ai, semiconductor, fab</t>
+          <t>openai, autonomous</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/openai-agent-goes-rogue-and-hacks-popular-ai-community-left-escape-plans-for-future-models-inside-the-companys-infrastructure</t>
+          <t>https://techcrunch.com/2026/07/26/hugging-face-ceo-calls-for-radical-transparency-after-unprecedented-openai-hack/</t>
         </is>
       </c>
     </row>
@@ -2132,34 +1880,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5.72</v>
+        <v>3.8</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>rec1.32+sig2.4+src1.2+corr0.8</t>
+          <t>rec2.0+sig0.6+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>AI cyberattacks mean we can't defend ourselves the same way as before: Singapore's founding cybersecurity chief</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>ai, nvidia, ai infrastructure, ai partnership</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>channelnewsasia.com</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.channelnewsasia.com/singapore/cybersecurity-csa-founding-chief-david-koh-ai-cyberattack-defend-6275631</t>
         </is>
       </c>
     </row>
@@ -2168,34 +1916,34 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4.79</v>
+        <v>3.68</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>rec1.59+sig1.2+src1.2+corr0.8</t>
+          <t>rec1.88+sig0.6+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>OpenAI agent goes rogue and hacks popular AI community — left escape plans for future models inside the company's infrastructure</t>
+          <t>Making sense of the panic over Chinese AI</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>openai, ai</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/openai-agent-goes-rogue-and-hacks-popular-ai-community-left-escape-plans-for-future-models-inside-the-companys-infrastructure</t>
+          <t>https://techcrunch.com/2026/07/26/making-sense-of-the-panic-over-chinese-ai/</t>
         </is>
       </c>
     </row>
@@ -2204,16 +1952,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4.1</v>
+        <v>3.67</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>rec2.3+sig0.6+src1.2+corr0.0</t>
+          <t>rec1.87+sig0.6+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>คอมพิวเตอร์ควอนตัม: เทคโนโลยีที่จะเปลี่ยนโลก หลังยุค AI</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2226,12 +1974,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>thansettakij.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>https://www.thansettakij.com/blogs/columnist/neotech-forums/664938</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
@@ -2240,21 +1988,21 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3.86</v>
+        <v>3.35</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>rec1.46+sig1.2+src1.2+corr0.0</t>
+          <t>rec0.95+sig1.2+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Grab an Nvidia RTX 5060 Ti gaming PC with Core Ultra 7 CPU and 32GB RAM for under $1,200 — Thermaltake's View u2660T-170 slashed by 33%</t>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>nvidia, amd</t>
+          <t>ai, nvidia</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -2267,7 +2015,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/pc-components/grab-an-nvidia-rtx-5060-ti-gaming-pc-with-core-ultra-7-cpu-and-32gb-ram-for-under-usd1-200-thermaltakes-view-u2660t-170-slashed-by-33-percent</t>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
@@ -2276,21 +2024,21 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>3.77</v>
+        <v>3.33</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>rec1.37+sig1.2+src1.2+corr0.0</t>
+          <t>rec1.53+sig0.6+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Samsung Elec wins $200 billion Broadcom AI chip partnership, boosting foundry push</t>
+          <t>TechCrunch Mobility: Uber bets on its former CEO</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>ai, chip</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -2298,12 +2046,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>reuters.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>https://www.reuters.com/business/autos-transportation/samsung-elec-wins-200-billion-broadcom-ai-chip-partnership-boosting-foundry-push-2026-07-25/</t>
+          <t>https://techcrunch.com/2026/07/26/techcrunch-mobility-uber-bets-on-its-former-ceo/</t>
         </is>
       </c>
     </row>
@@ -2312,21 +2060,21 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>3.71</v>
+        <v>3.14</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>rec0.11+sig2.4+src1.2+corr0.0</t>
+          <t>rec1.34+sig0.6+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Anthropic ออก Claude Opus 5 บอกเก่งเทียบเท่า Fable 5 แต่ถูกกว่าครึ่งหนึ่ง</t>
+          <t>How AI wealth could be distributed to all Americans</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>anthropic, claude, ปัญญาประดิษฐ์, โมเดล</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -2334,12 +2082,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>blognone.com</t>
+          <t>cnbc.com</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>https://www.blognone.com/node/151227</t>
+          <t>https://www.cnbc.com/amp/2026/07/26/how-can-ai-wealth-be-shared-with-all-americans.html</t>
         </is>
       </c>
     </row>
@@ -2348,21 +2096,21 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>3.65</v>
+        <v>3.08</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>rec1.25+sig1.2+src1.2+corr0.0</t>
+          <t>rec0.68+sig1.2+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>One fallen power line exposed a growing AI data center problem. Here’s how to fix it.</t>
+          <t>Meta AI อัปเดตความสามารถ ช่วยวางแผน สรุปเนื้อหา ด้วยโมเดล Muse Spark 1.1</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ai, data center</t>
+          <t>ai, โมเดล</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -2370,12 +2118,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/one-fallen-power-line-exposed-a-growing-ai-data-center-problem-heres-how-to-fix-it/</t>
+          <t>https://www.blognone.com/node/151235</t>
         </is>
       </c>
     </row>
@@ -2384,16 +2132,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>3.53</v>
+        <v>3.01</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>rec1.73+sig0.6+src1.2+corr0.0</t>
+          <t>rec1.21+sig0.6+src1.2+corr0.0</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>What is the AI Kill Switch Act proposed in the US and how will it work?</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2406,12 +2154,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>theverge.com</t>
+          <t>aljazeera.com</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+          <t>https://www.aljazeera.com/news/2026/7/26/what-is-the-ai-kill-switch-act-proposed-in-the-us-and-how-will-it-work</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2525,7 +2273,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>7.03</v>
+        <v>6.57</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2</v>
@@ -2542,7 +2290,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
@@ -2550,25 +2298,25 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>The homepage The Verge The Verge logo. Notifications Notifications Hamburger Navigation Button Navigation Drawer The Verge The Verge logo. Login / Sign Up close Close Light System Dark Subscribe Facebook Threads Instagram Youtube RSS Comments Drawer Notifications Comments Loading comments Getting the conversation ready... Tech Business News Google basically confirms the Pixel 11 is getting a price</t>
+          <t>The homepage The Verge The Verge logo. Notifications Notifications Hamburger Navigation Button Navigation Drawer The Verge The Verge logo. Login / Sign Up close Close Light System Dark Subscribe Facebook Threads Instagram Youtube RSS Comments Drawer Notifications Comments Loading comments Getting the conversation ready... Tech Gadgets News Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>google, apple, microsoft</t>
+          <t>apple, meta</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>5.8</v>
+        <v>4.4</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T14:13:36-04:00</t>
+          <t>2026-07-26T15:36:38-04:00</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -2578,30 +2326,30 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>7</v>
+        <v>6.1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>primary</t>
+          <t>citation</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>nvidianews.nvidia.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
@@ -2609,25 +2357,25 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>SK Group and NVIDIA Expand Strategic Partnership Across AI Factories and Next-Generation Memory</t>
+          <t>Can Apple make smart glasses that aren’t a constant privacy threat?</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Newsroom NVIDIA in Brief Exec Bios NVIDIA Blog Podcast Media Assets In the News Press Contacts Online Press Kits Press Release SHARE SK Group and NVIDIA Expand Strategic Partnership Across AI Factories and Next-Generation Memory $500-Billion-Plus NVIDIA-SK AI Initiative Spans SK Telecom’s AI Factory of up to 2 Gigawatts and SK hynix’s Long-Term AI Memory Partnership July 24, 2026 News Summary: SK </t>
+          <t xml:space="preserve">In Brief Posted: As Apple prepares to launch its first smart glasses, the company is also wrestling with how to address consumer privacy concerns, according to Bloomberg’s Mark Gurman . Gurman reports that Apple has pushed back the launch target from early 2027, with the glasses now set for unveiling at the Worldwide Developers Conference in June 2027 and actually becoming available by the end of </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>18.8</v>
+        <v>2.9</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 05:13:03 GMT</t>
+          <t>Sun, 26 Jul 2026 21:06:44 +0000</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -2637,13 +2385,13 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/sk-group-and-nvidia-expand-strategic-partnership-across-ai-factories-and-next-generation-memory</t>
+          <t>https://techcrunch.com/2026/07/26/can-apple-make-smart-glasses-that-arent-a-constant-privacy-threat/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>5.83</v>
+        <v>5.97</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2</v>
@@ -2660,7 +2408,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -2668,25 +2416,25 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>TECH BUSINESS NEWS Google basically confirms the Pixel 11 is getting a price hike It’s just the latest victim of RAMageddon. by Terrence O'Brien Jul 26, 2026, 1:13 AM GMT+7 5 5 Comments (All New) Image: Google Part Of RAM price hikes: the latest on the global memory shortage SEE ALL UPDATES Terrence O'Brien is the Verge’s weekend editor. He’s covered the tech industry for over 18 years and knows a</t>
+          <t>TECH GADGETS NEWS Apple is banking on privacy to set its smart glasses apart They’re expected be revealed next June at WWDC. by Terrence O'Brien Jul 27, 2026, 2:36 AM GMT+7 13 13 Comments (All New) Meta’s AI glasses have been the focus of controversy. Photo: Amelia Holowaty Krales / The Verge Terrence O'Brien is the Verge’s weekend editor. He’s covered the tech industry for over 18 years and knows</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>5.8</v>
+        <v>4.4</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 18:13:36 GMT</t>
+          <t>Sun, 26 Jul 2026 19:36:38 GMT</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -2696,13 +2444,13 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>5.42</v>
+        <v>5.79</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>2</v>
@@ -2714,12 +2462,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -2727,25 +2475,25 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>Apple's smart glasses delay reportedly stems in part from major privacy concerns</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Tom's Hardware Premium equips you with world-class coverage and detailed insights into the evolving hardware landscape. Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive i</t>
+          <t>The Apple team behind the upcoming smart glasses is reportedly exploring several tweaks related to user privacy. bluestork/Shutterstock Apple is expected to soon reveal its entry into the smart glasses market, but it may be taking its time to make sure it gets user privacy right. According to Bloomberg 's Mark Gurman, Apple is grappling with how to address major privacy concerns when it comes to s</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>10.1</v>
+        <v>6.3</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 13:55:35 +0000</t>
+          <t>Sun, 26 Jul 2026 17:43:38 +0000</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -2755,13 +2503,13 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.engadget.com/2223527/apple-smart-glasses-delay-major-privacy-concerns/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5.42</v>
+        <v>5.65</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2</v>
@@ -2786,25 +2534,25 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Tech Industry Artificial Intelligence Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories News By Anton Shilov Published 10 hours ago A lot of money, little to no details. (Image credit: Nvidia) Share this article 0 Join the conversation Follow us Add us as a preferred source on Google Newsletter Subscribe to o</t>
+          <t>Tom's Hardware Premium equips you with world-class coverage and detailed insights into the evolving hardware landscape. Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive i</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>nvidia, tesla</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>10.1</v>
+        <v>14</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 13:55:35 GMT</t>
+          <t>Sun, 26 Jul 2026 10:00:00 +0000</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -2814,16 +2562,16 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>5.36</v>
+        <v>5.65</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -2845,25 +2593,25 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Grab an Nvidia RTX 5060 Ti gaming PC with Core Ultra 7 CPU and 32GB RAM for under $1,200 — Thermaltake's View u2660T-170 slashed by 33%</t>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive into our proprietary testing data and compare hardware with detailed benchmarks. Go beyond the headlines with expert repo</t>
+          <t>PC Components GPUs AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second News By Mark Tyson Published 14 hours ago Now they have a total 32GB VRAM system on a budget, for local LLM inference. When you purchase through links on our site, we may earn an affiliate commission. Here’s how it works.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>amd, nvidia</t>
+          <t>nvidia, tesla</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>8.699999999999999</v>
+        <v>14</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 15:18:22 +0000</t>
+          <t>Sun, 26 Jul 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -2873,13 +2621,13 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/pc-components/grab-an-nvidia-rtx-5060-ti-gaming-pc-with-core-ultra-7-cpu-and-32gb-ram-for-under-usd1-200-thermaltakes-view-u2660t-170-slashed-by-33-percent</t>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>5.29</v>
+        <v>5.05</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1</v>
@@ -2891,12 +2639,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -2904,25 +2652,25 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. lawsuit accuses Amazon of illegally poaching executives</t>
+          <t>Here's our first look at Apple TV's Neuromancer adaptation</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>In Brief Posted: Warner Bros. Discovery filed a lawsuit this week accusing Amazon of interference with contractual relations, breach of contract, and unfair competition. As reported by Deadline , the lawsuit alleges Amazon has been “hurriedly seeking to pirate away a number of contracted employees,” including Pia Barlow, an HBO Max marketing executive who recently joined Amazon MGM Studios. Warner</t>
+          <t>We also now know when it will be released: January 22, 2027. Apple The Apple TV series based on William Gibson's genre-defining 1984 cyberpunk novel, Neuromancer, will hit the streaming platform on January 22 of next year. Apple dropped the news at San Diego Comic-Con this weekend alongside the first official teaser. Neuromancer stars Callum Turner, Briana Middleton, Mark Strong, Joseph Lee, Peter</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>3.1</v>
+        <v>5.6</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 20:55:11 +0000</t>
+          <t>Sun, 26 Jul 2026 18:25:03 +0000</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -2932,16 +2680,16 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/warner-bros-lawsuit-accuses-amazon-of-illegally-poaching-executives/</t>
+          <t>https://www.engadget.com/2223559/first-look-apple-tv-neuromancer-adaptation-teaser-trailer/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>5.22</v>
+        <v>4.9</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -2950,12 +2698,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>en.yna.co.kr</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -2963,25 +2711,25 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>(LEAD) Naver gets $10 bln investment from Nvidia, Brookfield</t>
+          <t>A new look for the Apple Watch may still be at least a year away</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Go to Contents Go to Navigation All Menu SEARCH History English Facebook Twitter RSS Feed Yonhap News Agency Today's date SUN. July 26, 2026 Today's weather Jeju31 ℃CAI Good 49 Seoul28 ℃CAI Good 30 Busan32 ℃CAI Good 42 Daegu30 ℃CAI Good 38 Incheon28 ℃CAI Good 30 Gwangju30 ℃CAI Good 26 Daejeon29 ℃CAI Good 41 Ulsan31 ℃CAI Good 30 Jeju31 ℃CAI Good 49 Seoul28 ℃CAI Good 30 Latest News (LEAD) Naver gets</t>
+          <t xml:space="preserve">Apple will refresh its Series 12 and Ultra 4 watches with better specs, but not a design overhaul. Apple The upcoming refreshes to the Apple Watch won't look much different from the existing models, but they will pack a lot more processing punch, according to the latest Bloomberg report. In the Power On newsletter, Mark Gurman reported that Apple is in "late-stage testing" for the refreshed Apple </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>12.2</v>
+        <v>7.2</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 11:46:27 GMT</t>
+          <t>Sun, 26 Jul 2026 16:45:27 +0000</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -2991,13 +2739,13 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>https://en.yna.co.kr/view/AEN20260725002051320</t>
+          <t>https://www.engadget.com/2223488/apple-watch-redesign-a-year-away-series-12-ultra-4-updates/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>5.15</v>
+        <v>4.79</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1</v>
@@ -3009,12 +2757,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -3022,25 +2770,25 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Elon Musk’s Boring Company reportedly raising funding at a $20 billion valuation</t>
+          <t>Carrie is just trying to make a friend in the new trailer</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">In Brief Posted: Elon Musk’s tunneling startup The Boring Company is in talks to raise a $4 billion funding round at a valuation of $20 billion, according to The Wall Street Journal . The deal hasn’t closed and the terms could change, the WSJ says. At $20 billion, the valuation would be a significant increase from The Boring Company’s $5.7 billion valuation in 2022 . The startup has already built </t>
+          <t xml:space="preserve">The homepage The Verge The Verge logo. Notifications Notifications Hamburger Navigation Button Navigation Drawer The Verge The Verge logo. Login / Sign Up close Close Light System Dark Subscribe Facebook Threads Instagram Youtube RSS Comments Drawer Notifications Comments Loading comments Getting the conversation ready... Entertainment News Comics Carrie is just trying to make a friend in the new </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>elon musk</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>4.6</v>
+        <v>8.4</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 19:23:32 +0000</t>
+          <t>2026-07-26T11:33:27-04:00</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -3050,13 +2798,13 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/elon-musks-boring-company-reportedly-raising-funding-at-a-20-billion-valuation/</t>
+          <t>https://www.theverge.com/entertainment/971069/carrie-amazon-mike-flanagan-trailer-comic-con</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>5</v>
+        <v>4.73</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1</v>
@@ -3068,7 +2816,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3081,25 +2829,25 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Microsoft shipped a native Xbox 360 emulator with its new backwards-compatible releases on PC — modders quickly got 360 games running with minor tweaks</t>
+          <t>You can get three months of Xbox Game Pass Ultimate for almost half off</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Tom's Hardware Premium equips you with world-class coverage and detailed insights into the evolving hardware landscape. Choose how you want to join Tom’s Hardware MEMBER Get started with free access to reviews, badges and discussions. Unlock exclusive tools and insights for enthusiasts who want more. Access Bench, Roadmaps, deep analysis and other exclusive tools. Bench Performance Database Dive i</t>
+          <t>The homepage The Verge The Verge logo. Notifications Notifications Hamburger Navigation Button Navigation Drawer The Verge The Verge logo. Login / Sign Up close Close Light System Dark Subscribe Facebook Threads Instagram Youtube RSS Comments Drawer Notifications Comments Loading comments Getting the conversation ready... Gadgets Gaming Verge Shopping You can get three months of Xbox Game Pass Ult</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>amd, microsoft</t>
+          <t>microsoft</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>12.5</v>
+        <v>9</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 11:30:00 +0000</t>
+          <t>2026-07-26T11:00:00-04:00</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -3109,13 +2857,13 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/video-games/xbox/microsoft-shipped-a-native-xbox-360-emulator-with-its-new-backwards-compatible-releases-on-pc-modders-quickly-got-360-games-running-with-minor-tweaks</t>
+          <t>https://www.theverge.com/gadgets/970775/xbox-game-pass-ultimate-deal-sale</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>4.93</v>
+        <v>4.68</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>1</v>
@@ -3132,7 +2880,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Meta Platforms</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -3140,25 +2888,25 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Meta walks back limits for its smart glasses' Conversation Focus feature, for now</t>
+          <t>Your Apple Watch calorie tracker is an educated guess, not a fact</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>A company spokesperson said that it’s “still exploring all our options for the best approach.” Meta If you're an owner of any of Meta's AI glasses , you should take advantage of the Conversation Focus feature while you can. As first reported by The Verge , Meta is pausing its rate limits for the accessibility feature that uses the glasses' speakers to amplify the voice of who you're talking to. Me</t>
+          <t>Accurately counting calories requires more data than a smartwatch can easily gather. Cherlynn Low for Engadget The Apple Watch has steadily improved year on year since its initial launch back in 2015. As much as we love the excellent Apple Watch Series 11 though, the Cupertino-based company's wearables aren't all that good at tracking the calories you burn on any given day. Plenty of Apple Watch a</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>6.9</v>
+        <v>9.5</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 17:08:31 +0000</t>
+          <t>Sun, 26 Jul 2026 14:30:00 +0000</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -3168,13 +2916,13 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>https://www.engadget.com/2223212/meta-walks-back-rate-limits-for-smart-glasses-conversation-focus/</t>
+          <t>https://www.engadget.com/2222496/apple-watch-heres-why-calorie-tracker-not-a-fact/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>4.9</v>
+        <v>4.59</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>1</v>
@@ -3186,7 +2934,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>livemint.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -3199,12 +2947,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Apple’s China chip gamble: Is it ready to bet on Pentagon-blacklisted CXMT and YMTC to win the AI race?</t>
+          <t>The reason why the MacBook Air doesn't need a fan</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Sun, Jul 26, 2026 SubscribeSign in E-Paper View Market Dashboard Home Markets News Mint Portfolio Premium Latest News IPO Companies Technology Money Mint Hindi More Apple’s China chip gamble: Is it ready to bet on Pentagon-blacklisted CXMT and YMTC to win the AI race? Sanchari Ghosh Updated 25 Jul 2026, 10:21 PM IST Apple claims suppliers are exploiting the market, leading to price increases on it</t>
+          <t xml:space="preserve">Apple Silicon delivers enough performance without overheating. Jonathan Weiss/Shutterstock Apple decided to ditch fans in the MacBook Air several years ago. The company made this significant hardware switch-up when it replaced Intel processors with its own silicon, starting with the M1 MacBook Air in late 2020. The main reason Apple was able to drop active cooling from its thinnest portable Macs? </t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -3213,11 +2961,11 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>7.2</v>
+        <v>10.5</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 16:48:00 GMT</t>
+          <t>Sun, 26 Jul 2026 13:30:00 +0000</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -3227,16 +2975,16 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>https://www.livemint.com/companies/news/apples-china-chip-gamble-is-it-ready-to-bet-on-pentagon-blacklisted-cxmt-and-ymtc-to-win-the-ai-race-11784993303522.html</t>
+          <t>https://www.engadget.com/2218722/macbook-air-missing-fan-reason-why/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>4.79</v>
+        <v>4.52</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -3245,7 +2993,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>koreaherald.com</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3258,12 +3006,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>'RAM Machine' case probably costs more than the entire build — Nvidia RTX 5060, Core Ultra 5 CPU, and 32GB DDR5-8200 RAM are hiding inside</t>
+          <t>KAIST, Nvidia deepen AI collaboration with joint research facilities</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Jowi Morales is a writer and journalist covering the tech beat since 2021. However, he’s been interested in technology far earlier than that. He started discovering desktop computers when his father brought home a Windows 95 PC, but his first real experience working under the hood of the PC was when</t>
+          <t>KAIST, Nvidia deepen AI collaboration with joint research facilities    The Korea Herald</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -3272,11 +3020,11 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>8.4</v>
+        <v>19.6</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 15:34:57 +0000</t>
+          <t>Sun, 26 Jul 2026 04:23:56 GMT</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -3286,13 +3034,13 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/desktops/gaming-pcs/ram-machine-case-probably-costs-more-than-the-entire-build-nvidia-rtx-5060-core-ultra-5-cpu-and-32gb-ddr5-8200-ram-are-hiding-inside</t>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE1raHBwX3I1Y21oZndZcXBOOWstNmpXbC1MSWpsSjVJSjhyeXdKMjJTTFJwMm1qLXVMc1MzWlpXUXNyVmp1YUxlLTNGaXY4dENLQVZPNXo1MA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>4.64</v>
+        <v>4.49</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>1</v>
@@ -3304,12 +3052,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>theverge.com</t>
+          <t>tomshardware.com</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -3317,25 +3065,25 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. is suing Amazon for poaching employees</t>
+          <t>XFX Radeon RX 9070 XT drops to its lowest price of the summer — save $90 on AMD's flagship RDNA 4 graphics card</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery has filed suit against Amazon, accusing it of  illegally poaching employees , including Pia Barlow, former senior VP for originals marketing. In the complaint, Warner says that "Amazon has chosen to ride on the coattails of other well-established Hollywood mainstays," and that</t>
+          <t>Kunal Khullar is a contributor at Tom’s Hardware with extensive writing experience in computing. With a deep-seated passion for technology, Kunal has dedicated years to mastering the intricacies of computer hardware components and staying at the forefront of the latest software developments. His jou</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>amd</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>9.9</v>
+        <v>11.5</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T10:05:12-04:00</t>
+          <t>Sun, 26 Jul 2026 12:31:14 +0000</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -3345,13 +3093,13 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/business/971011/warner-bros-suing-amazon-poaching-employees</t>
+          <t>https://www.tomshardware.com/pc-components/xfx-radeon-rx-9070-xt-drops-to-its-lowest-price-of-the-summer-save-usd90-on-amds-flagship-rdna-4-graphics-card</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>4.51</v>
+        <v>4.49</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>1</v>
@@ -3368,7 +3116,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -3376,25 +3124,25 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Delaware’s Printed Solid rebrands to Prusa USA</t>
+          <t>Minecraft system requirements raised for the first time in 17 years — Microsoft now recommends 16GB of RAM and a 2020s or newer CPU to run the Java Edition</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Denise has been crafting with PCs since she discovered Print Shop had clip art on her Apple IIe. She’s been a freelance newspaper reporter, online columnist and craft blogger with an eye for kid’s STEM activities. She got hooked on 3D printing after her son made a tiny Tinkercad Jeep for a school sc</t>
+          <t>Jowi Morales is a writer and journalist covering the tech beat since 2021. However, he’s been interested in technology far earlier than that. He started discovering desktop computers when his father brought home a Windows 95 PC, but his first real experience working under the hood of the PC was when</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>apple</t>
+          <t>microsoft</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>11.3</v>
+        <v>11.5</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 12:41:51 +0000</t>
+          <t>Sun, 26 Jul 2026 12:30:00 +0000</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -3404,7 +3152,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/3d-printing/delawares-printed-solid-rebrands-to-prusa-usa</t>
+          <t>https://www.tomshardware.com/video-games/pc-gaming/minecraft-system-requirements-raised-for-the-first-time-in-17-years-microsoft-now-recommends-16gb-of-ram-and-a-2020s-or-newer-cpu-to-run-the-java-edition</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3175,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -3435,18 +3183,19 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Folding and flipping phones are getting seriously good</t>
+          <t>The vertical video takeover is here</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Hi, friends! Welcome to  Installer  No. 137, your guide to the best and  Verge -iest stuff in the world. (If you're new here, welcome, happy phone season, and also you can read all the old editions at the   Installer  homepage .)  
- This week, I've been reading about   Google Zero   and   armored ca</t>
+          <t>This is   The Stepback  , a weekly newsletter breaking down one essential story from the tech world. For more on all things vertical video, follow    David Pierce  . The Stepback  arrives in our subscribers' inboxes on Sunday at 8AM ET. Opt in for  The Stepback   here .  
+ How it started 
+ For a whi</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
@@ -3454,7 +3203,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:00:00-04:00</t>
+          <t>2026-07-26T08:00:00-04:00</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -3464,30 +3213,30 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971004/z-fold8-xteink-x4-light-flip-installer</t>
+          <t>https://www.theverge.com/column/970756/vertical-video-tiktok-youtube-instagram-streaming-facebook</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>4.35</v>
+        <v>4.04</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>primary</t>
+          <t>citation</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>microsoft.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -3495,25 +3244,28 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Central Coast Council serves 355,000 citizens anytime, anywhere with Surface 5G</t>
+          <t>Meta ออกแอพแยก Seller สำหรับผู้ขายสินค้าบน Facebook Marketpace</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Central Coast Council serves 355,000 citizens anytime, anywhere with Surface 5G    Microsoft</t>
+          <t>Meta ออกแอพแยก Seller สำหรับผู้ขายสินค้าบน Facebook Marketpace 
+     Body 
+                Meta ออกแอพมือถือใหม่ชื่อ  Seller  เป็นแอพแยกสำหรับผู้ขายใน Facebook Marketplace 
+ Meta ให้เหตผลของการแยกแอพว่า ต้องการให้พื้นที่เฉพาะแก่ผู้ขาย มีเครื่องมืออำนวยความสะดวก เช่น สร้างรายละเอียดสินค้าด้วย AI</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>microsoft</t>
+          <t>facebook, meta</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>21.4</v>
+        <v>22.5</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 02:38:23 GMT</t>
+          <t>Sun, 26 Jul 2026 01:30:36 +0000</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -3523,30 +3275,30 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOV09YaGFWZldCbktTamVvSk5NSW9NRkJoY2h6X3Nta09CT1ZVTWhYZ1c1M09XTDlrLWdfR3l2SmpjNGZ4TUNZRENLMFQ2dkV1cVpBVTVGNEFxT1BQMTZJYXdEdU9Hb3Y4dWRmTFE1YlZTMjN4cUE1Tkd1Rm9saTJnT3VrMmZjQmM?oc=5</t>
+          <t>https://www.blognone.com/node/151231</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>4.34</v>
+        <v>3.98</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>screening</t>
+          <t>citation</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>asia.nikkei.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -3554,25 +3306,27 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Samsung, SK and Nvidia join $700bn US-Korea AI push</t>
+          <t>Meta AI อัปเดตความสามารถ ช่วยวางแผน สรุปเนื้อหา ด้วยโมเดล Muse Spark 1.1</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Samsung, SK and Nvidia join $700bn US-Korea AI push    Nikkei Asia</t>
+          <t>Meta AI อัปเดตความสามารถ ช่วยวางแผน สรุปเนื้อหา ด้วยโมเดล Muse Spark 1.1 
+     Body 
+                Meta AI แอปผู้ช่วย AI ของ Meta อัปเดตความสามารถใหม่หลังจากโมเดล [Muse Spark 1.1](Muse Spark 1.1) ออกมาเมื่อต้นเดือน โดยขยายความสามารถจากการเป็นแชทบอตถามตอบ ไปสู่ผู้ช่วยที่สามารถวางแผน คิด และให้</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>5.7</v>
+        <v>16.9</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 18:17:00 GMT</t>
+          <t>Sun, 26 Jul 2026 07:04:09 +0000</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -3582,13 +3336,13 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQWXlCbjAwQU9GTzVYS3hJaU5Xai1pYnE3XzZQU0N6Tkx5TXFXQ05wTkw3SDZ3RnNIV081RERZR2NYZHJzZG1mSXY3T2NWUXRVVDZwNG0zckdQSWVLUjMtdGNoblk0YTl6b0F3UF9VVE9IdmlQYWp2Y1VacUYzcGN4U0prNmowQkJfbmo0dHQwbEkySUEwQ0twN202SU9fUXJMdXlIMDRybVdnTkNVX19NOENjX3BJYVUw?oc=5</t>
+          <t>https://www.blognone.com/node/151235</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>4.26</v>
+        <v>3.88</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>1</v>
@@ -3600,38 +3354,38 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>engadget.com</t>
+          <t>tomshardware.com</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Amazon accused of poaching HBO employees in Warner Bros. lawsuit</t>
+          <t>Chinese CXMT DRAM doesn't look like the budget savior many were expecting — new modules enter the market, but prices still track the big three</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery has sued Amazon for 'inducing' its employees to breach their contracts.</t>
+          <t>Anton Shilov has been in the PC industry since 1990s playing games, building PCs, and writing stories about pretty much everything that relates to PCs, Macs, smartphones, tablets, and even fab equipment. Over his career, he has worked at a variety of high-ranking websites, including AnandTech, EE Ti</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>dram</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>13.9</v>
+        <v>10.6</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 10:08:37 +0000</t>
+          <t>Sun, 26 Jul 2026 13:25:30 +0000</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -3641,13 +3395,13 @@
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>https://www.engadget.com/2223135/amazon-accused-poaching-hbo-employees-warner-bros-lawsuit/</t>
+          <t>https://www.tomshardware.com/pc-components/dram/chinese-cxmt-dram-doesnt-look-like-the-budget-savior-many-were-expecting-new-modules-enter-the-market-but-prices-still-track-the-big-three</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>4.2</v>
+        <v>3.46</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>1</v>
@@ -3659,38 +3413,40 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Kalshi demands Netflix take down trailer for ‘Prediction Games’ documentary</t>
+          <t>Facebook ออกแบดจ์ Facebook Verified ยืนยันว่ามีตัวตน ด้วยการสแกนใบหน้า</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Kalshi claims the trailer is “defamatory” and contains “both fabricated documents and false and misleading statements.”</t>
+          <t>Facebook ออกแบดจ์ Facebook Verified ยืนยันว่ามีตัวตน ด้วยการสแกนใบหน้า 
+     Body 
+                Facebook ประกาศเพิ่มบริการใหม่ให้แบดจ์เครื่องติ๊กถูกแบบไม่มีสีฟ้า เรียกชื่อว่า  Facebook Verified  โดยการได้เครื่องหมายดังกล่าว ผู้ใช้งานต้องสแกนใบหน้าผ่านระบบของ Facebook เพื่อเทียบกับรูปในโปรไฟล</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>netflix</t>
+          <t>facebook</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>7.2</v>
+        <v>22.3</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 16:46:46 +0000</t>
+          <t>Sun, 26 Jul 2026 01:40:54 +0000</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -3700,13 +3456,13 @@
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/kalshi-demands-netflix-take-down-trailer-for-prediction-games-documentary/</t>
+          <t>https://www.blognone.com/node/151232</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>3.78</v>
+        <v>3.41</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>1</v>
@@ -3718,12 +3474,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>cnbc.com</t>
+          <t>koreaherald.com</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -3731,25 +3487,25 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Nvidia locks down memory supply from SK Hynix as part of $500 billion AI deal</t>
+          <t>Samsung bets on lighter AI glasses to challenge Meta</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Nvidia locks down memory supply from SK Hynix as part of $500 billion AI deal    CNBC</t>
+          <t>Samsung bets on lighter AI glasses to challenge Meta    The Korea Herald</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>19</v>
+        <v>22.8</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Sat, 25 Jul 2026 05:00:01 GMT</t>
+          <t>Sun, 26 Jul 2026 01:10:27 GMT</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -3759,309 +3515,12 @@
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNbXdIVGF2aEhFZkd2RUt4cWJPYnRleXU3VVAwQmdzeFhkVFVLSTduM0FuUFhrR052VGNpLVAzLXo4cHo0NTM0NUR3bG94RGowSDFwZ2E2SjZHTG1SM3M1TVU4bkVJSTZteUc5U3JGZ0ZNTGpfamo2UEpfbk9Jdk9hbHVrMC0zUU9ITmdyNTY3VWtvejRRX282N0packdXaDRKeVRjOGhiTUR5d9IBrwFBVV95cUxQMlAtRUpKdjI3MjdkS0JIckxFdGY2MzVxSVN1eWVPMFFHLXVNUF9teGt1SXZPWG9XU24xZTdpUFk2V183UXdUSXE2SnUyR2NfbXBLX0dlOF96VE8wRXd6ekg3QkVJajlPcEE5Z18teXJ4dko3MktYelZmb1BlbGJjRU5ueTlkZ19CbUlMRnJaWVdXd2NjZ2l1VnVsenNJYng3bVVxdkp0bEV6LXg0ZnNz?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>livemint.com</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>AI News Tracker: An Open AI agent goes rogue, while Amazon plans AI unit layoffs</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>AI News Tracker: An Open AI agent goes rogue, while Amazon plans AI unit layoffs    livemint.com</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>amazon</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 03:30:38 GMT</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYXNWWmRRSzRyelpRVDJMbjhrbFBYeEJuRkpwTGZtNjhJYmtOM3VQc0hrdTAyUGJQUGdZUVRXU0hTdXRjYUs0aDk4aklJZjRFRVk4cldsYXZSdUtDeHp5Y0JGV1R1QU95RzEtd3RTbTVtUnlpaW0yLXpWU0dYOWcwT1F1MEU3aTlETXZvaExUX0VZR0tWMjZac0E1Z0xmVUJiZlFlWnl0bklfV3RnSVZlYnhLRHhlYnFHOWhTOHB4RmpvNHhKOGhKMlNfa9IB0AFBVV95cUxQMDl3MFNPbkRzNnVKeGZGVk8tNjRPREpsR2dtZ293MHdzM1VNOG94amRjS1NTSkF1eXkyUTBodTF0anlSYWVETGR5X3d6VmtvMG1JQTg1WEpHM3B6cmF5cGkzRW1OVGRYcHZNWVQxNUJHTjlRYmlEUk1udExpOTRYUElkSU1rcmpkYmZuX2Iyb1JNcGM5NFYwQjNDbzFrWjNfSkxyYk5aR2sycHdkWE5mWE1wc1RiNHFPc19oZnAwd04yWThtWE5uQXZHZi1MWFFn?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>aljazeera.com</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Alphabet</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Trump threatens EU will pay ‘big price’ after Brussels fines Google $1bn</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Trump threatens EU will pay ‘big price’ after Brussels fines Google $1bn    Al Jazeera</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="n">
-        <v>22.6</v>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 01:21:25 GMT</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="M24" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQSkM0dWJiQ19hZWthNHlFVWN5QVFPNTdkaHpybFFGQXF2VklzWFRpazFYV3dJOFE0TjdKWkVabWVpWXN5dWxrclJHaVlMUnFiREo3djNRRmROWHE2QUFlNVFxTTZTek01VkE0QzlaUG5fOVR2dlNHcllNNF9vVGRxNHpBNzBiN2hZOWdUQnZrYUF5QmhEQmlSQ0QyUWJXR0d6dEt0ZWVzYlo2dFg5U3A40gG0AUFVX3lxTE5aU3A0VHEyUUZaaVNGMmxGZmxzYVBReld6M2xKMEI4b19TYTBYRnhrM3R5ZGR5NUdaM0FtSEs3NlNGVFk1Z0xORUdmWGRyaTV4LTZfVXVRQWF2bWFLelI5ekduSlRQSTh5b2hHUFI2NVVBdG04aEJ4anJpRXRiREhYQU54VzR4UFA1QXdROHltY21KLW90YUE4Q0ROTmUwdE1NYjljVXotQ1RFR2NyV21acDk3RQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>citation</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>blognone.com</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Anthropic ออก Claude Opus 5 บอกเก่งเทียบเท่า Fable 5 แต่ถูกกว่าครึ่งหนึ่ง</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Anthropic ออก Claude Opus 5 บอกเก่งเทียบเท่า Fable 5 แต่ถูกกว่าครึ่งหนึ่ง 
-     Body 
-                Anthropic อัปเดตโมเดลปัญญาประดิษฐ์รุ่น(เคย)บน  Claude Opus 5  โดยคราวนี้เทียบกับ Fable 5 ที่เป็นโมเดลรุ่นบนสุดปัจจุบัน บอกว่ามีความฉลาดในการทำงานซับซ้อนใกล้เคียงกัน แต่ราคาใช้งานถูกกว่าครึ่งหนึ</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>anthropic</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="n">
-        <v>22.9</v>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 01:07:52 +0000</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="inlineStr">
-        <is>
-          <t>https://www.blognone.com/node/151227</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>screening</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>bloomberg.com</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Nvidia</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Watch Nvidia CEO Jensen Huang on the AI Boom in South Korea</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Watch Nvidia CEO Jensen Huang on the AI Boom in South Korea    Bloomberg.com</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>jensen huang, nvidia</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 00:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWXR6SW90a016T3VnSzdrNWtGLTg2UDBHYUVzWld1bXRzeXlDVmttLUtPOWxMQjlNU3o1VmRtX2NvNVdKMnN6eVotVTJfbUhjRG1ScEhWWUxVLWpJajlwUUNnTkFOZWI1cXdaaUZINWpGNEZOMVFkUFlNdnp1WUVUUUtjWl9kdGdvbk9JUUNIY2lfWW9OUmF3X3dHcnRCODVqejhTOW9VRGZSNlo4?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>screening</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>theinformation.com</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Nvidia</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Nvidia Forms $500 Billion AI ‘Partnership’ With Memory Chip Giant SK</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Nvidia Forms $500 Billion AI ‘Partnership’ With Memory Chip Giant SK    The Information</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>nvidia</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Sat, 25 Jul 2026 05:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>skipped</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQVkIycWY4WF9Nc19nRDV4SDFQbnQ1TVpld3J0WHVGelpfdnZBN0Nya3NWb2ZUMHNlMUhqZWpXZlc1SXBFSFVWaUtqN1NFeWNZTnZPd2xLcjVCY3FGRU13bjNzNE9Zb0JsQlh4Q3pyelNWcWwwdjdaVzFHWXBzN1BmWUl6NDZvd1dtMHNicTFaenZwWXRsV2RXU3ZkR0YtX3RBQXpJ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTFBUWERRdmtrY1dhT1BCRVp4ZkNDYXRpOWRFZVNhUHlteVRpUkFQTFpiRjM5WnZubHN2Nm5WWmRoczg4anpkV1liY05tdTFFb2lvMFhBSzBDQQ?oc=5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M27"/>
+  <autoFilter ref="A1:M22"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -4084,11 +3543,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4166,26 +3620,26 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>7.03</v>
+        <v>6.57</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>rec1.73+sig1.8+src1.2+corr0.8+wl1.5</t>
+          <t>rec1.87+sig1.2+src1.2+corr0.8+wl1.5</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>google, apple, microsoft</t>
+          <t>apple, meta</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
@@ -4198,7 +3652,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
@@ -4207,39 +3661,39 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>7</v>
+        <v>6.1</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>rec0.5+sig0.6+src2.0+corr2.4+wl1.5</t>
+          <t>rec2.0+sig0.6+src1.2+corr0.8+wl1.5</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>SK Group and NVIDIA Expand Strategic Partnership Across AI Factories and Next-Generation Memory</t>
+          <t>Can Apple make smart glasses that aren’t a constant privacy threat?</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>nvidianews.nvidia.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/sk-group-and-nvidia-expand-strategic-partnership-across-ai-factories-and-next-generation-memory</t>
+          <t>https://techcrunch.com/2026/07/26/can-apple-make-smart-glasses-that-arent-a-constant-privacy-threat/</t>
         </is>
       </c>
     </row>
@@ -4248,26 +3702,26 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5.83</v>
+        <v>5.97</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>rec1.73+sig0.6+src1.2+corr0.8+wl1.5</t>
+          <t>rec1.87+sig0.6+src1.2+corr0.8+wl1.5</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Alphabet</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
@@ -4280,7 +3734,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
@@ -4289,26 +3743,26 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>5.42</v>
+        <v>5.79</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>rec1.32+sig0.6+src1.2+corr0.8+wl1.5</t>
+          <t>rec1.69+sig0.6+src1.2+corr0.8+wl1.5</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>Apple's smart glasses delay reportedly stems in part from major privacy concerns</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
@@ -4316,12 +3770,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.engadget.com/2223527/apple-smart-glasses-delay-major-privacy-concerns/</t>
         </is>
       </c>
     </row>
@@ -4330,16 +3784,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>5.42</v>
+        <v>5.65</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>rec1.32+sig0.6+src1.2+corr0.8+wl1.5</t>
+          <t>rec0.95+sig1.2+src1.2+corr0.8+wl1.5</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -4349,7 +3803,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>nvidia, tesla</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
@@ -4362,7 +3816,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
@@ -4371,16 +3825,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>5.36</v>
+        <v>5.65</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>rec1.46+sig1.2+src1.2+corr0.0+wl1.5</t>
+          <t>rec0.95+sig1.2+src1.2+corr0.8+wl1.5</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Grab an Nvidia RTX 5060 Ti gaming PC with Core Ultra 7 CPU and 32GB RAM for under $1,200 — Thermaltake's View u2660T-170 slashed by 33%</t>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -4390,11 +3844,11 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>amd, nvidia</t>
+          <t>nvidia, tesla</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -4403,7 +3857,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/pc-components/grab-an-nvidia-rtx-5060-ti-gaming-pc-with-core-ultra-7-cpu-and-32gb-ram-for-under-usd1-200-thermaltakes-view-u2660t-170-slashed-by-33-percent</t>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
@@ -4412,26 +3866,26 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>5.29</v>
+        <v>5.05</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>rec1.99+sig0.6+src1.2+corr0.0+wl1.5</t>
+          <t>rec1.75+sig0.6+src1.2+corr0.0+wl1.5</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. lawsuit accuses Amazon of illegally poaching executives</t>
+          <t>Here's our first look at Apple TV's Neuromancer adaptation</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
@@ -4439,12 +3893,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/warner-bros-lawsuit-accuses-amazon-of-illegally-poaching-executives/</t>
+          <t>https://www.engadget.com/2223559/first-look-apple-tv-neuromancer-adaptation-teaser-trailer/</t>
         </is>
       </c>
     </row>
@@ -4453,39 +3907,39 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>5.22</v>
+        <v>4.9</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>rec1.12+sig0.6+src1.2+corr0.8+wl1.5</t>
+          <t>rec1.6+sig0.6+src1.2+corr0.0+wl1.5</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>(LEAD) Naver gets $10 bln investment from Nvidia, Brookfield</t>
+          <t>A new look for the Apple Watch may still be at least a year away</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>en.yna.co.kr</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>https://en.yna.co.kr/view/AEN20260725002051320</t>
+          <t>https://www.engadget.com/2223488/apple-watch-redesign-a-year-away-series-12-ultra-4-updates/</t>
         </is>
       </c>
     </row>
@@ -4494,26 +3948,26 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>5.15</v>
+        <v>4.79</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>rec1.85+sig0.6+src1.2+corr0.0+wl1.5</t>
+          <t>rec1.49+sig0.6+src1.2+corr0.0+wl1.5</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Elon Musk’s Boring Company reportedly raising funding at a $20 billion valuation</t>
+          <t>Carrie is just trying to make a friend in the new trailer</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Tesla</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>elon musk</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -4521,12 +3975,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/elon-musks-boring-company-reportedly-raising-funding-at-a-20-billion-valuation/</t>
+          <t>https://www.theverge.com/entertainment/971069/carrie-amazon-mike-flanagan-trailer-comic-con</t>
         </is>
       </c>
     </row>
@@ -4535,16 +3989,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>5</v>
+        <v>4.73</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>rec1.1+sig1.2+src1.2+corr0.0+wl1.5</t>
+          <t>rec1.43+sig0.6+src1.2+corr0.0+wl1.5</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Microsoft shipped a native Xbox 360 emulator with its new backwards-compatible releases on PC — modders quickly got 360 games running with minor tweaks</t>
+          <t>You can get three months of Xbox Game Pass Ultimate for almost half off</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -4554,7 +4008,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>amd, microsoft</t>
+          <t>microsoft</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
@@ -4562,12 +4016,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/video-games/xbox/microsoft-shipped-a-native-xbox-360-emulator-with-its-new-backwards-compatible-releases-on-pc-modders-quickly-got-360-games-running-with-minor-tweaks</t>
+          <t>https://www.theverge.com/gadgets/970775/xbox-game-pass-ultimate-deal-sale</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4613,576 +4067,469 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Nvidia  (Tier 1 · 10 stories)</t>
+          <t>Apple  (Tier 1 · 8 stories)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>7</v>
+        <v>6.57</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SK Group and NVIDIA Expand Strategic Partnership Across AI Factories and Next-Generation Memory</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>nvidianews.nvidia.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>https://nvidianews.nvidia.com/news/sk-group-and-nvidia-expand-strategic-partnership-across-ai-factories-and-next-generation-memory</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>5.42</v>
+        <v>6.1</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>Can Apple make smart glasses that aren’t a constant privacy threat?</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>techcrunch.com</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://techcrunch.com/2026/07/26/can-apple-make-smart-glasses-that-arent-a-constant-privacy-threat/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5.42</v>
+        <v>5.97</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Nvidia and SK Group enter $500 billion AI partnership — plan to supercharge AI infrastructure with next-gen memory and massive AI factories</t>
+          <t>Apple is banking on privacy to set its smart glasses apart</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/tech-industry/artificial-intelligence/nvidia-and-sk-group-enter-usd500-billion-ai-partnership-plan-to-supercharge-ai-infrastructure-with-next-gen-memory-and-massive-ai-factories</t>
+          <t>https://www.theverge.com/tech/971101/apple-smart-glasses-privacy</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>5.36</v>
+        <v>5.79</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Grab an Nvidia RTX 5060 Ti gaming PC with Core Ultra 7 CPU and 32GB RAM for under $1,200 — Thermaltake's View u2660T-170 slashed by 33%</t>
+          <t>Apple's smart glasses delay reportedly stems in part from major privacy concerns</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/pc-components/grab-an-nvidia-rtx-5060-ti-gaming-pc-with-core-ultra-7-cpu-and-32gb-ram-for-under-usd1-200-thermaltakes-view-u2660t-170-slashed-by-33-percent</t>
+          <t>https://www.engadget.com/2223527/apple-smart-glasses-delay-major-privacy-concerns/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>5.22</v>
+        <v>5.05</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>(LEAD) Naver gets $10 bln investment from Nvidia, Brookfield</t>
+          <t>Here's our first look at Apple TV's Neuromancer adaptation</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>en.yna.co.kr</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>https://en.yna.co.kr/view/AEN20260725002051320</t>
+          <t>https://www.engadget.com/2223559/first-look-apple-tv-neuromancer-adaptation-teaser-trailer/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>4.79</v>
+        <v>4.9</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>'RAM Machine' case probably costs more than the entire build — Nvidia RTX 5060, Core Ultra 5 CPU, and 32GB DDR5-8200 RAM are hiding inside</t>
+          <t>A new look for the Apple Watch may still be at least a year away</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>tomshardware.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>https://www.tomshardware.com/desktops/gaming-pcs/ram-machine-case-probably-costs-more-than-the-entire-build-nvidia-rtx-5060-core-ultra-5-cpu-and-32gb-ddr5-8200-ram-are-hiding-inside</t>
+          <t>https://www.engadget.com/2223488/apple-watch-redesign-a-year-away-series-12-ultra-4-updates/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>4.34</v>
+        <v>4.68</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Samsung, SK and Nvidia join $700bn US-Korea AI push</t>
+          <t>Your Apple Watch calorie tracker is an educated guess, not a fact</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>asia.nikkei.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxQWXlCbjAwQU9GTzVYS3hJaU5Xai1pYnE3XzZQU0N6Tkx5TXFXQ05wTkw3SDZ3RnNIV081RERZR2NYZHJzZG1mSXY3T2NWUXRVVDZwNG0zckdQSWVLUjMtdGNoblk0YTl6b0F3UF9VVE9IdmlQYWp2Y1VacUYzcGN4U0prNmowQkJfbmo0dHQwbEkySUEwQ0twN202SU9fUXJMdXlIMDRybVdnTkNVX19NOENjX3BJYVUw?oc=5</t>
+          <t>https://www.engadget.com/2222496/apple-watch-heres-why-calorie-tracker-not-a-fact/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>3.78</v>
+        <v>4.59</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Nvidia locks down memory supply from SK Hynix as part of $500 billion AI deal</t>
+          <t>The reason why the MacBook Air doesn't need a fan</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>cnbc.com</t>
+          <t>engadget.com</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxNbXdIVGF2aEhFZkd2RUt4cWJPYnRleXU3VVAwQmdzeFhkVFVLSTduM0FuUFhrR052VGNpLVAzLXo4cHo0NTM0NUR3bG94RGowSDFwZ2E2SjZHTG1SM3M1TVU4bkVJSTZteUc5U3JGZ0ZNTGpfamo2UEpfbk9Jdk9hbHVrMC0zUU9ITmdyNTY3VWtvejRRX282N0packdXaDRKeVRjOGhiTUR5d9IBrwFBVV95cUxQMlAtRUpKdjI3MjdkS0JIckxFdGY2MzVxSVN1eWVPMFFHLXVNUF9teGt1SXZPWG9XU24xZTdpUFk2V183UXdUSXE2SnUyR2NfbXBLX0dlOF96VE8wRXd6ekg3QkVJajlPcEE5Z18teXJ4dko3MktYelZmb1BlbGJjRU5ueTlkZ19CbUlMRnJaWVdXd2NjZ2l1VnVsenNJYng3bVVxdkp0bEV6LXg0ZnNz?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Watch Nvidia CEO Jensen Huang on the AI Boom in South Korea</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>bloomberg.com</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPWXR6SW90a016T3VnSzdrNWtGLTg2UDBHYUVzWld1bXRzeXlDVmttLUtPOWxMQjlNU3o1VmRtX2NvNVdKMnN6eVotVTJfbUhjRG1ScEhWWUxVLWpJajlwUUNnTkFOZWI1cXdaaUZINWpGNEZOMVFkUFlNdnp1WUVUUUtjWl9kdGdvbk9JUUNIY2lfWW9OUmF3X3dHcnRCODVqejhTOW9VRGZSNlo4?oc=5</t>
+          <t>https://www.engadget.com/2218722/macbook-air-missing-fan-reason-why/</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Nvidia Forms $500 Billion AI ‘Partnership’ With Memory Chip Giant SK</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>theinformation.com</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxQVkIycWY4WF9Nc19nRDV4SDFQbnQ1TVpld3J0WHVGelpfdnZBN0Nya3NWb2ZUMHNlMUhqZWpXZlc1SXBFSFVWaUtqN1NFeWNZTnZPd2xLcjVCY3FGRU13bjNzNE9Zb0JsQlh4Q3pyelNWcWwwdjdaVzFHWXBzN1BmWUl6NDZvd1dtMHNicTFaenZwWXRsV2RXU3ZkR0YtX3RBQXpJ?oc=5</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Meta Platforms  (Tier 1 · 5 stories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>The vertical video takeover is here</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>theverge.com</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.theverge.com/column/970756/vertical-video-tiktok-youtube-instagram-streaming-facebook</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Amazon  (Tier 1 · 5 stories)</t>
+      <c r="A15" s="2" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Meta ออกแอพแยก Seller สำหรับผู้ขายสินค้าบน Facebook Marketpace</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>blognone.com</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.blognone.com/node/151231</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>5.29</v>
+        <v>3.98</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. lawsuit accuses Amazon of illegally poaching executives</t>
+          <t>Meta AI อัปเดตความสามารถ ช่วยวางแผน สรุปเนื้อหา ด้วยโมเดล Muse Spark 1.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>techcrunch.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/07/25/warner-bros-lawsuit-accuses-amazon-of-illegally-poaching-executives/</t>
+          <t>https://www.blognone.com/node/151235</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>4.64</v>
+        <v>3.46</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. is suing Amazon for poaching employees</t>
+          <t>Facebook ออกแบดจ์ Facebook Verified ยืนยันว่ามีตัวตน ด้วยการสแกนใบหน้า</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>theverge.com</t>
+          <t>blognone.com</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/business/971011/warner-bros-suing-amazon-poaching-employees</t>
+          <t>https://www.blognone.com/node/151232</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>4.26</v>
+        <v>3.41</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Amazon accused of poaching HBO employees in Warner Bros. lawsuit</t>
+          <t>Samsung bets on lighter AI glasses to challenge Meta</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>engadget.com</t>
+          <t>koreaherald.com</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>https://www.engadget.com/2223135/amazon-accused-poaching-hbo-employees-warner-bros-lawsuit/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>AI News Tracker: An Open AI agent goes rogue, while Amazon plans AI unit layoffs</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>livemint.com</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOYXNWWmRRSzRyelpRVDJMbjhrbFBYeEJuRkpwTGZtNjhJYmtOM3VQc0hrdTAyUGJQUGdZUVRXU0hTdXRjYUs0aDk4aklJZjRFRVk4cldsYXZSdUtDeHp5Y0JGV1R1QU95RzEtd3RTbTVtUnlpaW0yLXpWU0dYOWcwT1F1MEU3aTlETXZvaExUX0VZR0tWMjZac0E1Z0xmVUJiZlFlWnl0bklfV3RnSVZlYnhLRHhlYnFHOWhTOHB4RmpvNHhKOGhKMlNfa9IB0AFBVV95cUxQMDl3MFNPbkRzNnVKeGZGVk8tNjRPREpsR2dtZ293MHdzM1VNOG94amRjS1NTSkF1eXkyUTBodTF0anlSYWVETGR5X3d6VmtvMG1JQTg1WEpHM3B6cmF5cGkzRW1OVGRYcHZNWVQxNUJHTjlRYmlEUk1udExpOTRYUElkSU1rcmpkYmZuX2Iyb1JNcGM5NFYwQjNDbzFrWjNfSkxyYk5aR2sycHdkWE5mWE1wc1RiNHFPc19oZnAwd04yWThtWE5uQXZHZi1MWFFn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTFBUWERRdmtrY1dhT1BCRVp4ZkNDYXRpOWRFZVNhUHlteVRpUkFQTFpiRjM5WnZubHN2Nm5WWmRoczg4anpkV1liY05tdTFFb2lvMFhBSzBDQQ?oc=5</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Anthropic ออก Claude Opus 5 บอกเก่งเทียบเท่า Fable 5 แต่ถูกกว่าครึ่งหนึ่ง</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>blognone.com</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>https://www.blognone.com/node/151227</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Nvidia  (Tier 1 · 3 stories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>tomshardware.com</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Alphabet  (Tier 1 · 3 stories)</t>
+      <c r="A22" s="2" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>AI enthusiast adds Nvidia Tesla V100 as loud as a lawnmower to gaming PC for $266 — 32GB of VRAM rig can run 27 billion parameter model at 32 tokens per second</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>tomshardware.com</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/pc-components/gpus/ai-enthusiast-adds-nvidia-tesla-v100-as-loud-as-a-lawnmower-to-gaming-pc-for-usd266-32gb-of-vram-rig-can-run-27-billion-parameter-model-at-32-tokens-per-second</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>5.83</v>
+        <v>4.52</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
+          <t>KAIST, Nvidia deepen AI collaboration with joint research facilities</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
+          <t>koreaherald.com</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE1raHBwX3I1Y21oZndZcXBOOWstNmpXbC1MSWpsSjVJSjhyeXdKMjJTTFJwMm1qLXVMc1MzWlpXUXNyVmp1YUxlLTNGaXY4dENLQVZPNXo1MA?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Microsoft  (Tier 1 · 2 stories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>You can get three months of Xbox Game Pass Ultimate for almost half off</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
           <t>theverge.com</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Folding and flipping phones are getting seriously good</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>theverge.com</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>https://www.theverge.com/tech/971004/z-fold8-xteink-x4-light-flip-installer</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Trump threatens EU will pay ‘big price’ after Brussels fines Google $1bn</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>aljazeera.com</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxQSkM0dWJiQ19hZWthNHlFVWN5QVFPNTdkaHpybFFGQXF2VklzWFRpazFYV3dJOFE0TjdKWkVabWVpWXN5dWxrclJHaVlMUnFiREo3djNRRmROWHE2QUFlNVFxTTZTek01VkE0QzlaUG5fOVR2dlNHcllNNF9vVGRxNHpBNzBiN2hZOWdUQnZrYUF5QmhEQmlSQ0QyUWJXR0d6dEt0ZWVzYlo2dFg5U3A40gG0AUFVX3lxTE5aU3A0VHEyUUZaaVNGMmxGZmxzYVBReld6M2xKMEI4b19TYTBYRnhrM3R5ZGR5NUdaM0FtSEs3NlNGVFk1Z0xORUdmWGRyaTV4LTZfVXVRQWF2bWFLelI5ekduSlRQSTh5b2hHUFI2NVVBdG04aEJ4anJpRXRiREhYQU54VzR4UFA1QXdROHltY21KLW90YUE4Q0ROTmUwdE1NYjljVXotQ1RFR2NyV21acDk3RQ?oc=5</t>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.theverge.com/gadgets/970775/xbox-game-pass-ultimate-deal-sale</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Microsoft  (Tier 1 · 3 stories)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>7.03</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Google basically confirms the Pixel 11 is getting a price hike</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>theverge.com</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>https://www.theverge.com/tech/971041/google-confirms-pixel-11-price-hike</t>
+      <c r="A27" s="2" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Minecraft system requirements raised for the first time in 17 years — Microsoft now recommends 16GB of RAM and a 2020s or newer CPU to run the Java Edition</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>tomshardware.com</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/video-games/pc-gaming/minecraft-system-requirements-raised-for-the-first-time-in-17-years-microsoft-now-recommends-16gb-of-ram-and-a-2020s-or-newer-cpu-to-run-the-java-edition</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Microsoft shipped a native Xbox 360 emulator with its new backwards-compatible releases on PC — modders quickly got 360 games running with minor tweaks</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>tomshardware.com</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>https://www.tomshardware.com/video-games/xbox/microsoft-shipped-a-native-xbox-360-emulator-with-its-new-backwards-compatible-releases-on-pc-modders-quickly-got-360-games-running-with-minor-tweaks</t>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>AMD  (Tier 1 · 1 stories)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>4.35</v>
+        <v>4.49</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Central Coast Council serves 355,000 citizens anytime, anywhere with Surface 5G</t>
+          <t>XFX Radeon RX 9070 XT drops to its lowest price of the summer — save $90 on AMD's flagship RDNA 4 graphics card</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>microsoft.com</t>
+          <t>tomshardware.com</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxOV09YaGFWZldCbktTamVvSk5NSW9NRkJoY2h6X3Nta09CT1ZVTWhYZ1c1M09XTDlrLWdfR3l2SmpjNGZ4TUNZRENLMFQ2dkV1cVpBVTVGNEFxT1BQMTZJYXdEdU9Hb3Y4dWRmTFE1YlZTMjN4cUE1Tkd1Rm9saTJnT3VrMmZjQmM?oc=5</t>
+          <t>https://www.tomshardware.com/pc-components/xfx-radeon-rx-9070-xt-drops-to-its-lowest-price-of-the-summer-save-usd90-on-amds-flagship-rdna-4-graphics-card</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Apple  (Tier 1 · 2 stories)</t>
+          <t>Amazon  (Tier 1 · 1 stories)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>4.9</v>
+        <v>4.79</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Apple’s China chip gamble: Is it ready to bet on Pentagon-blacklisted CXMT and YMTC to win the AI race?</t>
+          <t>Carrie is just trying to make a friend in the new trailer</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>livemint.com</t>
+          <t>theverge.com</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>https://www.livemint.com/companies/news/apples-china-chip-gamble-is-it-ready-to-bet-on-pentagon-blacklisted-cxmt-and-ymtc-to-win-the-ai-race-11784993303522.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>4.51</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Delaware’s Printed Solid rebrands to Prusa USA</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
+          <t>https://www.theverge.com/entertainment/971069/carrie-amazon-mike-flanagan-trailer-comic-con</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Micron Technology  (Tier 2 · 1 stories)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Chinese CXMT DRAM doesn't look like the budget savior many were expecting — new modules enter the market, but prices still track the big three</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>tomshardware.com</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>https://www.tomshardware.com/3d-printing/delawares-printed-solid-rebrands-to-prusa-usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Meta Platforms  (Tier 1 · 1 stories)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>4.93</v>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Meta walks back limits for its smart glasses' Conversation Focus feature, for now</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>engadget.com</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>https://www.engadget.com/2223212/meta-walks-back-rate-limits-for-smart-glasses-conversation-focus/</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Tesla  (Tier 1 · 1 stories)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Elon Musk’s Boring Company reportedly raising funding at a $20 billion valuation</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>techcrunch.com</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>https://techcrunch.com/2026/07/25/elon-musks-boring-company-reportedly-raising-funding-at-a-20-billion-valuation/</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Netflix  (Tier 2 · 1 stories)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Kalshi demands Netflix take down trailer for ‘Prediction Games’ documentary</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>techcrunch.com</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>https://techcrunch.com/2026/07/25/kalshi-demands-netflix-take-down-trailer-for-prediction-games-documentary/</t>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/pc-components/dram/chinese-cxmt-dram-doesnt-look-like-the-budget-savior-many-were-expecting-new-modules-enter-the-market-but-prices-still-track-the-big-three</t>
         </is>
       </c>
     </row>
@@ -5196,24 +4543,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>